<commit_message>
Drukmeting consistent over alle documenten; 09b versie 1.3 lean
09b 1.3: op basis van Janou's bewerking herschikt (eenmalig, dan de meting
in volgorde, achtergrond achteraan), verantwoording en bronnummers uit de
tekst, doelregio's volgens het manuscript (hiel alleen bij vorige
voetzweer), rol van eCRF 24b. Pressure Monitoring Tool: blad Visit en
sjabloon naar acht regio's (codes A-P), pedar-zolen als figuur, hielregel;
tool nu ook in Per visite V1/V2/V4/V6/V8. eCRF 24b: hielregel.
Referentie visite 2 i.p.v. "dezelfde sessie" in manuscript, doctoraatsplan,
opleidingsplanning, WP1-afvinklijst, Groeninge- en congresdeck (+ scripts),
werkpakket1-tijdlijn. Toestemmingsformulier (eCRF 02 x3, model-ICF): meting
in de schoen, beide armen gemeten, herhaling op maand 6/12/18. REDCap:
drie snelheidsvelden weg (1410 velden), toelichting referentie. Geen
netwerkdatabase. PARADISE_BRONNEN bijgewerkt.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/(e)CRF/Per nummer/24b_Opvolgtool piekdruk en ontlasting (Novel pedar).xlsx
+++ b/(e)CRF/Per nummer/24b_Opvolgtool piekdruk en ontlasting (Novel pedar).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://kuleuven-my.sharepoint.com/personal/janou_debuyser_kuleuven_be1/Documents/Documents/PhD Brugge/Site/(e)CRF/Per nummer/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="7" documentId="11_71D650B1929CCFA6FD70D0ED0D1FF050D6CE9E36" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2FBA11EF-3AEA-412D-B272-78A02FCB2FB8}"/>
+  <xr:revisionPtr revIDLastSave="24" documentId="11_71D650B1929CCFA6FD70D0ED0D1FF050D6CE9E36" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DC9D05F0-9D7A-487C-BCAA-544881AB70D2}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -146,18 +146,18 @@
     <t>RECHTS - regio van de vorige voetzweer:</t>
   </si>
   <si>
-    <t>De doelregio's zijn de regio van de vorige voetzweer - altijd, ook onder 200 kPa, gekozen bovenaan bij elke voet - aangevuld met de een of twee regio's met de hoogste piekdruk zonder zool op visite 2. Beide worden automatisch als DOELREGIO gemarkeerd.
+    <t>Schermafbeelding van het MPP-beeld (novel studio)</t>
+  </si>
+  <si>
+    <t>Plak hieronder de schermafbeelding van het MPP-beeld, met de kleurenschaal erbij, voor de visite die bovenaan staat. Windows + Shift + S om te knippen, Ctrl + V om te plakken; de afbeelding mag het gearceerde vak overlappen.</t>
+  </si>
+  <si>
+    <t>[ plak hier de schermafbeelding van het MPP-beeld ]</t>
+  </si>
+  <si>
+    <t>Doelregio's per voet: de regio van de vorige voetzweer - altijd, ook onder 200 kPa - plus de twee regio's in voorvoet of middenvoet met de hoogste piekdruk boven 200 kPa zonder zool. De hiel telt alleen mee als daar de vorige voetzweer zat. Beide worden automatisch als DOELREGIO gemarkeerd; de vorige voetzweer kies je bovenaan bij elke voet.
 Norm per doelregio: piekdruk met zool onder 200 kPa, OF minstens 25% lager dan de referentie. De referentie is de meting zonder zool op visite 2 (in-shoe, in hetzelfde schoeisel, zonder de CMFO) en blijft op visite 4, 6 en 8 dezelfde. Noteer op visite 2 de waarde na de laatste aanpassing.
 Is de norm niet gehaald (NEE), of kleurt een piekdruk oranje omdat ze 5% of meer hoger ligt dan de vorige visite, dan wordt de CMFO aangepast volgens eCRF 23 en opnieuw gemeten.</t>
-  </si>
-  <si>
-    <t>Schermafbeelding van het MPP-beeld (novel studio)</t>
-  </si>
-  <si>
-    <t>Plak hieronder de schermafbeelding van het MPP-beeld, met de kleurenschaal erbij, voor de visite die bovenaan staat. Windows + Shift + S om te knippen, Ctrl + V om te plakken; de afbeelding mag het gearceerde vak overlappen.</t>
-  </si>
-  <si>
-    <t>[ plak hier de schermafbeelding van het MPP-beeld ]</t>
   </si>
 </sst>
 </file>
@@ -472,11 +472,26 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -489,27 +504,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standaard" xfId="0" builtinId="0"/>
@@ -568,6 +568,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -875,7 +879,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="25" t="s">
+      <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="10"/>
@@ -894,7 +898,7 @@
       <c r="O1" s="10"/>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A2" s="22" t="s">
+      <c r="A2" s="18" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="10"/>
@@ -978,16 +982,16 @@
       </c>
     </row>
     <row r="12" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="11" t="s">
+      <c r="A12" s="15" t="s">
         <v>31</v>
       </c>
-      <c r="B12" s="11"/>
-      <c r="C12" s="11"/>
-      <c r="D12" s="11"/>
-      <c r="E12" s="29"/>
-      <c r="F12" s="29"/>
-      <c r="G12" s="29"/>
-      <c r="H12" s="30" t="s">
+      <c r="B12" s="15"/>
+      <c r="C12" s="15"/>
+      <c r="D12" s="15"/>
+      <c r="E12" s="16"/>
+      <c r="F12" s="16"/>
+      <c r="G12" s="16"/>
+      <c r="H12" s="17" t="s">
         <v>32</v>
       </c>
       <c r="I12" s="10"/>
@@ -999,7 +1003,7 @@
       <c r="O12" s="10"/>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A13" s="21"/>
+      <c r="A13" s="19"/>
       <c r="B13" s="10"/>
       <c r="C13" s="10"/>
       <c r="D13" s="10"/>
@@ -1016,31 +1020,31 @@
       <c r="O13" s="10"/>
     </row>
     <row r="14" spans="1:15" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="9" t="s">
+      <c r="A14" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="B14" s="9" t="s">
+      <c r="B14" s="14" t="s">
         <v>33</v>
       </c>
-      <c r="C14" s="9" t="s">
+      <c r="C14" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="D14" s="9" t="s">
+      <c r="D14" s="14" t="s">
         <v>16</v>
       </c>
       <c r="E14" s="10"/>
       <c r="F14" s="10"/>
-      <c r="G14" s="9" t="s">
+      <c r="G14" s="14" t="s">
         <v>17</v>
       </c>
       <c r="H14" s="10"/>
       <c r="I14" s="10"/>
-      <c r="J14" s="9" t="s">
+      <c r="J14" s="14" t="s">
         <v>18</v>
       </c>
       <c r="K14" s="10"/>
       <c r="L14" s="10"/>
-      <c r="M14" s="9" t="s">
+      <c r="M14" s="14" t="s">
         <v>19</v>
       </c>
       <c r="N14" s="10"/>
@@ -1093,7 +1097,7 @@
       </c>
       <c r="B16" s="5"/>
       <c r="C16" s="6" t="str">
-        <f>IF($E$12=$A16,"DOELREGIO",IF(B16="","",IF(AND(B16&gt;200,RANK(B16,$B$16:$B$23)&lt;=2),"DOELREGIO","")))</f>
+        <f>IF($E$12=$A16,"DOELREGIO","")</f>
         <v/>
       </c>
       <c r="D16" s="5"/>
@@ -1139,7 +1143,7 @@
       </c>
       <c r="B17" s="5"/>
       <c r="C17" s="6" t="str">
-        <f>IF($E$12=$A17,"DOELREGIO",IF(B17="","",IF(AND(B17&gt;200,RANK(B17,$B$16:$B$23)&lt;=2),"DOELREGIO","")))</f>
+        <f>IF($E$12=$A17,"DOELREGIO",IF(B17="","",IF(AND(B17&gt;200,RANK(B17,$B$17:$B$23)&lt;=2),"DOELREGIO","")))</f>
         <v/>
       </c>
       <c r="D17" s="5"/>
@@ -1185,7 +1189,7 @@
       </c>
       <c r="B18" s="5"/>
       <c r="C18" s="6" t="str">
-        <f>IF($E$12=$A18,"DOELREGIO",IF(B18="","",IF(AND(B18&gt;200,RANK(B18,$B$16:$B$23)&lt;=2),"DOELREGIO","")))</f>
+        <f>IF($E$12=$A18,"DOELREGIO",IF(B18="","",IF(AND(B18&gt;200,RANK(B18,$B$17:$B$23)&lt;=2),"DOELREGIO","")))</f>
         <v/>
       </c>
       <c r="D18" s="5"/>
@@ -1231,7 +1235,7 @@
       </c>
       <c r="B19" s="5"/>
       <c r="C19" s="6" t="str">
-        <f>IF($E$12=$A19,"DOELREGIO",IF(B19="","",IF(AND(B19&gt;200,RANK(B19,$B$16:$B$23)&lt;=2),"DOELREGIO","")))</f>
+        <f>IF($E$12=$A19,"DOELREGIO",IF(B19="","",IF(AND(B19&gt;200,RANK(B19,$B$17:$B$23)&lt;=2),"DOELREGIO","")))</f>
         <v/>
       </c>
       <c r="D19" s="5"/>
@@ -1277,7 +1281,7 @@
       </c>
       <c r="B20" s="5"/>
       <c r="C20" s="6" t="str">
-        <f>IF($E$12=$A20,"DOELREGIO",IF(B20="","",IF(AND(B20&gt;200,RANK(B20,$B$16:$B$23)&lt;=2),"DOELREGIO","")))</f>
+        <f>IF($E$12=$A20,"DOELREGIO",IF(B20="","",IF(AND(B20&gt;200,RANK(B20,$B$17:$B$23)&lt;=2),"DOELREGIO","")))</f>
         <v/>
       </c>
       <c r="D20" s="5"/>
@@ -1323,7 +1327,7 @@
       </c>
       <c r="B21" s="5"/>
       <c r="C21" s="6" t="str">
-        <f>IF($E$12=$A21,"DOELREGIO",IF(B21="","",IF(AND(B21&gt;200,RANK(B21,$B$16:$B$23)&lt;=2),"DOELREGIO","")))</f>
+        <f>IF($E$12=$A21,"DOELREGIO",IF(B21="","",IF(AND(B21&gt;200,RANK(B21,$B$17:$B$23)&lt;=2),"DOELREGIO","")))</f>
         <v/>
       </c>
       <c r="D21" s="5"/>
@@ -1369,7 +1373,7 @@
       </c>
       <c r="B22" s="5"/>
       <c r="C22" s="6" t="str">
-        <f>IF($E$12=$A22,"DOELREGIO",IF(B22="","",IF(AND(B22&gt;200,RANK(B22,$B$16:$B$23)&lt;=2),"DOELREGIO","")))</f>
+        <f>IF($E$12=$A22,"DOELREGIO",IF(B22="","",IF(AND(B22&gt;200,RANK(B22,$B$17:$B$23)&lt;=2),"DOELREGIO","")))</f>
         <v/>
       </c>
       <c r="D22" s="5"/>
@@ -1415,7 +1419,7 @@
       </c>
       <c r="B23" s="5"/>
       <c r="C23" s="6" t="str">
-        <f>IF($E$12=$A23,"DOELREGIO",IF(B23="","",IF(AND(B23&gt;200,RANK(B23,$B$16:$B$23)&lt;=2),"DOELREGIO","")))</f>
+        <f>IF($E$12=$A23,"DOELREGIO",IF(B23="","",IF(AND(B23&gt;200,RANK(B23,$B$17:$B$23)&lt;=2),"DOELREGIO","")))</f>
         <v/>
       </c>
       <c r="D23" s="5"/>
@@ -1456,16 +1460,16 @@
       </c>
     </row>
     <row r="25" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="11" t="s">
+      <c r="A25" s="15" t="s">
         <v>36</v>
       </c>
-      <c r="B25" s="11"/>
-      <c r="C25" s="11"/>
-      <c r="D25" s="11"/>
-      <c r="E25" s="29"/>
-      <c r="F25" s="29"/>
-      <c r="G25" s="29"/>
-      <c r="H25" s="30" t="s">
+      <c r="B25" s="15"/>
+      <c r="C25" s="15"/>
+      <c r="D25" s="15"/>
+      <c r="E25" s="16"/>
+      <c r="F25" s="16"/>
+      <c r="G25" s="16"/>
+      <c r="H25" s="17" t="s">
         <v>32</v>
       </c>
       <c r="I25" s="10"/>
@@ -1477,7 +1481,7 @@
       <c r="O25" s="10"/>
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A26" s="21"/>
+      <c r="A26" s="19"/>
       <c r="B26" s="10"/>
       <c r="C26" s="10"/>
       <c r="D26" s="10"/>
@@ -1494,31 +1498,31 @@
       <c r="O26" s="10"/>
     </row>
     <row r="27" spans="1:15" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="9" t="s">
+      <c r="A27" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="B27" s="9" t="s">
+      <c r="B27" s="14" t="s">
         <v>33</v>
       </c>
-      <c r="C27" s="9" t="s">
+      <c r="C27" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="D27" s="9" t="s">
+      <c r="D27" s="14" t="s">
         <v>16</v>
       </c>
       <c r="E27" s="10"/>
       <c r="F27" s="10"/>
-      <c r="G27" s="9" t="s">
+      <c r="G27" s="14" t="s">
         <v>17</v>
       </c>
       <c r="H27" s="10"/>
       <c r="I27" s="10"/>
-      <c r="J27" s="9" t="s">
+      <c r="J27" s="14" t="s">
         <v>18</v>
       </c>
       <c r="K27" s="10"/>
       <c r="L27" s="10"/>
-      <c r="M27" s="9" t="s">
+      <c r="M27" s="14" t="s">
         <v>19</v>
       </c>
       <c r="N27" s="10"/>
@@ -1571,7 +1575,7 @@
       </c>
       <c r="B29" s="5"/>
       <c r="C29" s="6" t="str">
-        <f>IF($E$25=$A29,"DOELREGIO",IF(B29="","",IF(AND(B29&gt;200,RANK(B29,$B$29:$B$36)&lt;=2),"DOELREGIO","")))</f>
+        <f>IF($E$25=$A29,"DOELREGIO","")</f>
         <v/>
       </c>
       <c r="D29" s="5"/>
@@ -1617,7 +1621,7 @@
       </c>
       <c r="B30" s="5"/>
       <c r="C30" s="6" t="str">
-        <f>IF($E$25=$A30,"DOELREGIO",IF(B30="","",IF(AND(B30&gt;200,RANK(B30,$B$29:$B$36)&lt;=2),"DOELREGIO","")))</f>
+        <f>IF($E$25=$A30,"DOELREGIO",IF(B30="","",IF(AND(B30&gt;200,RANK(B30,$B$30:$B$36)&lt;=2),"DOELREGIO","")))</f>
         <v/>
       </c>
       <c r="D30" s="5"/>
@@ -1663,7 +1667,7 @@
       </c>
       <c r="B31" s="5"/>
       <c r="C31" s="6" t="str">
-        <f>IF($E$25=$A31,"DOELREGIO",IF(B31="","",IF(AND(B31&gt;200,RANK(B31,$B$29:$B$36)&lt;=2),"DOELREGIO","")))</f>
+        <f>IF($E$25=$A31,"DOELREGIO",IF(B31="","",IF(AND(B31&gt;200,RANK(B31,$B$30:$B$36)&lt;=2),"DOELREGIO","")))</f>
         <v/>
       </c>
       <c r="D31" s="5"/>
@@ -1709,7 +1713,7 @@
       </c>
       <c r="B32" s="5"/>
       <c r="C32" s="6" t="str">
-        <f>IF($E$25=$A32,"DOELREGIO",IF(B32="","",IF(AND(B32&gt;200,RANK(B32,$B$29:$B$36)&lt;=2),"DOELREGIO","")))</f>
+        <f>IF($E$25=$A32,"DOELREGIO",IF(B32="","",IF(AND(B32&gt;200,RANK(B32,$B$30:$B$36)&lt;=2),"DOELREGIO","")))</f>
         <v/>
       </c>
       <c r="D32" s="5"/>
@@ -1755,7 +1759,7 @@
       </c>
       <c r="B33" s="5"/>
       <c r="C33" s="6" t="str">
-        <f>IF($E$25=$A33,"DOELREGIO",IF(B33="","",IF(AND(B33&gt;200,RANK(B33,$B$29:$B$36)&lt;=2),"DOELREGIO","")))</f>
+        <f>IF($E$25=$A33,"DOELREGIO",IF(B33="","",IF(AND(B33&gt;200,RANK(B33,$B$30:$B$36)&lt;=2),"DOELREGIO","")))</f>
         <v/>
       </c>
       <c r="D33" s="5"/>
@@ -1801,7 +1805,7 @@
       </c>
       <c r="B34" s="5"/>
       <c r="C34" s="6" t="str">
-        <f>IF($E$25=$A34,"DOELREGIO",IF(B34="","",IF(AND(B34&gt;200,RANK(B34,$B$29:$B$36)&lt;=2),"DOELREGIO","")))</f>
+        <f>IF($E$25=$A34,"DOELREGIO",IF(B34="","",IF(AND(B34&gt;200,RANK(B34,$B$30:$B$36)&lt;=2),"DOELREGIO","")))</f>
         <v/>
       </c>
       <c r="D34" s="5"/>
@@ -1847,7 +1851,7 @@
       </c>
       <c r="B35" s="5"/>
       <c r="C35" s="6" t="str">
-        <f>IF($E$25=$A35,"DOELREGIO",IF(B35="","",IF(AND(B35&gt;200,RANK(B35,$B$29:$B$36)&lt;=2),"DOELREGIO","")))</f>
+        <f>IF($E$25=$A35,"DOELREGIO",IF(B35="","",IF(AND(B35&gt;200,RANK(B35,$B$30:$B$36)&lt;=2),"DOELREGIO","")))</f>
         <v/>
       </c>
       <c r="D35" s="5"/>
@@ -1893,7 +1897,7 @@
       </c>
       <c r="B36" s="5"/>
       <c r="C36" s="6" t="str">
-        <f>IF($E$25=$A36,"DOELREGIO",IF(B36="","",IF(AND(B36&gt;200,RANK(B36,$B$29:$B$36)&lt;=2),"DOELREGIO","")))</f>
+        <f>IF($E$25=$A36,"DOELREGIO",IF(B36="","",IF(AND(B36&gt;200,RANK(B36,$B$30:$B$36)&lt;=2),"DOELREGIO","")))</f>
         <v/>
       </c>
       <c r="D36" s="5"/>
@@ -1934,7 +1938,7 @@
       </c>
     </row>
     <row r="39" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="23" t="s">
+      <c r="A39" s="29" t="s">
         <v>29</v>
       </c>
       <c r="B39" s="10"/>
@@ -1953,8 +1957,8 @@
       <c r="O39" s="10"/>
     </row>
     <row r="40" spans="1:15" ht="90" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="24" t="s">
-        <v>37</v>
+      <c r="A40" s="30" t="s">
+        <v>40</v>
       </c>
       <c r="B40" s="10"/>
       <c r="C40" s="10"/>
@@ -2006,8 +2010,8 @@
       <c r="O42" s="10"/>
     </row>
     <row r="44" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="23" t="s">
-        <v>38</v>
+      <c r="A44" s="29" t="s">
+        <v>37</v>
       </c>
       <c r="B44" s="10"/>
       <c r="C44" s="10"/>
@@ -2026,7 +2030,7 @@
     </row>
     <row r="45" spans="1:15" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="20" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B45" s="10"/>
       <c r="C45" s="10"/>
@@ -2061,26 +2065,26 @@
       <c r="O46" s="10"/>
     </row>
     <row r="48" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A48" s="12" t="s">
-        <v>40</v>
-      </c>
-      <c r="B48" s="13"/>
-      <c r="C48" s="13"/>
-      <c r="D48" s="13"/>
-      <c r="E48" s="13"/>
-      <c r="F48" s="13"/>
-      <c r="G48" s="13"/>
-      <c r="H48" s="13"/>
-      <c r="I48" s="13"/>
-      <c r="J48" s="13"/>
-      <c r="K48" s="13"/>
-      <c r="L48" s="13"/>
-      <c r="M48" s="13"/>
-      <c r="N48" s="13"/>
-      <c r="O48" s="14"/>
+      <c r="A48" s="21" t="s">
+        <v>39</v>
+      </c>
+      <c r="B48" s="22"/>
+      <c r="C48" s="22"/>
+      <c r="D48" s="22"/>
+      <c r="E48" s="22"/>
+      <c r="F48" s="22"/>
+      <c r="G48" s="22"/>
+      <c r="H48" s="22"/>
+      <c r="I48" s="22"/>
+      <c r="J48" s="22"/>
+      <c r="K48" s="22"/>
+      <c r="L48" s="22"/>
+      <c r="M48" s="22"/>
+      <c r="N48" s="22"/>
+      <c r="O48" s="23"/>
     </row>
     <row r="49" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A49" s="15"/>
+      <c r="A49" s="24"/>
       <c r="B49" s="10"/>
       <c r="C49" s="10"/>
       <c r="D49" s="10"/>
@@ -2094,10 +2098,10 @@
       <c r="L49" s="10"/>
       <c r="M49" s="10"/>
       <c r="N49" s="10"/>
-      <c r="O49" s="16"/>
+      <c r="O49" s="25"/>
     </row>
     <row r="50" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A50" s="15"/>
+      <c r="A50" s="24"/>
       <c r="B50" s="10"/>
       <c r="C50" s="10"/>
       <c r="D50" s="10"/>
@@ -2111,10 +2115,10 @@
       <c r="L50" s="10"/>
       <c r="M50" s="10"/>
       <c r="N50" s="10"/>
-      <c r="O50" s="16"/>
+      <c r="O50" s="25"/>
     </row>
     <row r="51" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A51" s="15"/>
+      <c r="A51" s="24"/>
       <c r="B51" s="10"/>
       <c r="C51" s="10"/>
       <c r="D51" s="10"/>
@@ -2128,10 +2132,10 @@
       <c r="L51" s="10"/>
       <c r="M51" s="10"/>
       <c r="N51" s="10"/>
-      <c r="O51" s="16"/>
+      <c r="O51" s="25"/>
     </row>
     <row r="52" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A52" s="15"/>
+      <c r="A52" s="24"/>
       <c r="B52" s="10"/>
       <c r="C52" s="10"/>
       <c r="D52" s="10"/>
@@ -2145,10 +2149,10 @@
       <c r="L52" s="10"/>
       <c r="M52" s="10"/>
       <c r="N52" s="10"/>
-      <c r="O52" s="16"/>
+      <c r="O52" s="25"/>
     </row>
     <row r="53" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A53" s="15"/>
+      <c r="A53" s="24"/>
       <c r="B53" s="10"/>
       <c r="C53" s="10"/>
       <c r="D53" s="10"/>
@@ -2162,10 +2166,10 @@
       <c r="L53" s="10"/>
       <c r="M53" s="10"/>
       <c r="N53" s="10"/>
-      <c r="O53" s="16"/>
+      <c r="O53" s="25"/>
     </row>
     <row r="54" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A54" s="15"/>
+      <c r="A54" s="24"/>
       <c r="B54" s="10"/>
       <c r="C54" s="10"/>
       <c r="D54" s="10"/>
@@ -2179,10 +2183,10 @@
       <c r="L54" s="10"/>
       <c r="M54" s="10"/>
       <c r="N54" s="10"/>
-      <c r="O54" s="16"/>
+      <c r="O54" s="25"/>
     </row>
     <row r="55" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A55" s="15"/>
+      <c r="A55" s="24"/>
       <c r="B55" s="10"/>
       <c r="C55" s="10"/>
       <c r="D55" s="10"/>
@@ -2196,10 +2200,10 @@
       <c r="L55" s="10"/>
       <c r="M55" s="10"/>
       <c r="N55" s="10"/>
-      <c r="O55" s="16"/>
+      <c r="O55" s="25"/>
     </row>
     <row r="56" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A56" s="15"/>
+      <c r="A56" s="24"/>
       <c r="B56" s="10"/>
       <c r="C56" s="10"/>
       <c r="D56" s="10"/>
@@ -2213,10 +2217,10 @@
       <c r="L56" s="10"/>
       <c r="M56" s="10"/>
       <c r="N56" s="10"/>
-      <c r="O56" s="16"/>
+      <c r="O56" s="25"/>
     </row>
     <row r="57" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A57" s="15"/>
+      <c r="A57" s="24"/>
       <c r="B57" s="10"/>
       <c r="C57" s="10"/>
       <c r="D57" s="10"/>
@@ -2230,10 +2234,10 @@
       <c r="L57" s="10"/>
       <c r="M57" s="10"/>
       <c r="N57" s="10"/>
-      <c r="O57" s="16"/>
+      <c r="O57" s="25"/>
     </row>
     <row r="58" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A58" s="15"/>
+      <c r="A58" s="24"/>
       <c r="B58" s="10"/>
       <c r="C58" s="10"/>
       <c r="D58" s="10"/>
@@ -2247,10 +2251,10 @@
       <c r="L58" s="10"/>
       <c r="M58" s="10"/>
       <c r="N58" s="10"/>
-      <c r="O58" s="16"/>
+      <c r="O58" s="25"/>
     </row>
     <row r="59" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A59" s="15"/>
+      <c r="A59" s="24"/>
       <c r="B59" s="10"/>
       <c r="C59" s="10"/>
       <c r="D59" s="10"/>
@@ -2264,10 +2268,10 @@
       <c r="L59" s="10"/>
       <c r="M59" s="10"/>
       <c r="N59" s="10"/>
-      <c r="O59" s="16"/>
+      <c r="O59" s="25"/>
     </row>
     <row r="60" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A60" s="15"/>
+      <c r="A60" s="24"/>
       <c r="B60" s="10"/>
       <c r="C60" s="10"/>
       <c r="D60" s="10"/>
@@ -2281,10 +2285,10 @@
       <c r="L60" s="10"/>
       <c r="M60" s="10"/>
       <c r="N60" s="10"/>
-      <c r="O60" s="16"/>
+      <c r="O60" s="25"/>
     </row>
     <row r="61" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A61" s="15"/>
+      <c r="A61" s="24"/>
       <c r="B61" s="10"/>
       <c r="C61" s="10"/>
       <c r="D61" s="10"/>
@@ -2298,10 +2302,10 @@
       <c r="L61" s="10"/>
       <c r="M61" s="10"/>
       <c r="N61" s="10"/>
-      <c r="O61" s="16"/>
+      <c r="O61" s="25"/>
     </row>
     <row r="62" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A62" s="15"/>
+      <c r="A62" s="24"/>
       <c r="B62" s="10"/>
       <c r="C62" s="10"/>
       <c r="D62" s="10"/>
@@ -2315,10 +2319,10 @@
       <c r="L62" s="10"/>
       <c r="M62" s="10"/>
       <c r="N62" s="10"/>
-      <c r="O62" s="16"/>
+      <c r="O62" s="25"/>
     </row>
     <row r="63" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A63" s="15"/>
+      <c r="A63" s="24"/>
       <c r="B63" s="10"/>
       <c r="C63" s="10"/>
       <c r="D63" s="10"/>
@@ -2332,10 +2336,10 @@
       <c r="L63" s="10"/>
       <c r="M63" s="10"/>
       <c r="N63" s="10"/>
-      <c r="O63" s="16"/>
+      <c r="O63" s="25"/>
     </row>
     <row r="64" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A64" s="15"/>
+      <c r="A64" s="24"/>
       <c r="B64" s="10"/>
       <c r="C64" s="10"/>
       <c r="D64" s="10"/>
@@ -2349,10 +2353,10 @@
       <c r="L64" s="10"/>
       <c r="M64" s="10"/>
       <c r="N64" s="10"/>
-      <c r="O64" s="16"/>
+      <c r="O64" s="25"/>
     </row>
     <row r="65" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A65" s="15"/>
+      <c r="A65" s="24"/>
       <c r="B65" s="10"/>
       <c r="C65" s="10"/>
       <c r="D65" s="10"/>
@@ -2366,10 +2370,10 @@
       <c r="L65" s="10"/>
       <c r="M65" s="10"/>
       <c r="N65" s="10"/>
-      <c r="O65" s="16"/>
+      <c r="O65" s="25"/>
     </row>
     <row r="66" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A66" s="15"/>
+      <c r="A66" s="24"/>
       <c r="B66" s="10"/>
       <c r="C66" s="10"/>
       <c r="D66" s="10"/>
@@ -2383,10 +2387,10 @@
       <c r="L66" s="10"/>
       <c r="M66" s="10"/>
       <c r="N66" s="10"/>
-      <c r="O66" s="16"/>
+      <c r="O66" s="25"/>
     </row>
     <row r="67" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A67" s="15"/>
+      <c r="A67" s="24"/>
       <c r="B67" s="10"/>
       <c r="C67" s="10"/>
       <c r="D67" s="10"/>
@@ -2400,10 +2404,10 @@
       <c r="L67" s="10"/>
       <c r="M67" s="10"/>
       <c r="N67" s="10"/>
-      <c r="O67" s="16"/>
+      <c r="O67" s="25"/>
     </row>
     <row r="68" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A68" s="15"/>
+      <c r="A68" s="24"/>
       <c r="B68" s="10"/>
       <c r="C68" s="10"/>
       <c r="D68" s="10"/>
@@ -2417,36 +2421,51 @@
       <c r="L68" s="10"/>
       <c r="M68" s="10"/>
       <c r="N68" s="10"/>
-      <c r="O68" s="16"/>
+      <c r="O68" s="25"/>
     </row>
     <row r="69" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A69" s="17"/>
-      <c r="B69" s="18"/>
-      <c r="C69" s="18"/>
-      <c r="D69" s="18"/>
-      <c r="E69" s="18"/>
-      <c r="F69" s="18"/>
-      <c r="G69" s="18"/>
-      <c r="H69" s="18"/>
-      <c r="I69" s="18"/>
-      <c r="J69" s="18"/>
-      <c r="K69" s="18"/>
-      <c r="L69" s="18"/>
-      <c r="M69" s="18"/>
-      <c r="N69" s="18"/>
-      <c r="O69" s="19"/>
+      <c r="A69" s="26"/>
+      <c r="B69" s="27"/>
+      <c r="C69" s="27"/>
+      <c r="D69" s="27"/>
+      <c r="E69" s="27"/>
+      <c r="F69" s="27"/>
+      <c r="G69" s="27"/>
+      <c r="H69" s="27"/>
+      <c r="I69" s="27"/>
+      <c r="J69" s="27"/>
+      <c r="K69" s="27"/>
+      <c r="L69" s="27"/>
+      <c r="M69" s="27"/>
+      <c r="N69" s="27"/>
+      <c r="O69" s="28"/>
     </row>
     <row r="71" spans="1:15" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A71" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="C71" s="26"/>
-      <c r="D71" s="27"/>
-      <c r="E71" s="27"/>
-      <c r="F71" s="28"/>
+      <c r="C71" s="11"/>
+      <c r="D71" s="12"/>
+      <c r="E71" s="12"/>
+      <c r="F71" s="13"/>
     </row>
   </sheetData>
   <mergeCells count="31">
+    <mergeCell ref="A48:O69"/>
+    <mergeCell ref="A45:O46"/>
+    <mergeCell ref="A44:O44"/>
+    <mergeCell ref="A39:O39"/>
+    <mergeCell ref="A40:O42"/>
+    <mergeCell ref="C27:C28"/>
+    <mergeCell ref="J14:L14"/>
+    <mergeCell ref="G27:I27"/>
+    <mergeCell ref="B14:B15"/>
+    <mergeCell ref="A3:O3"/>
+    <mergeCell ref="A27:A28"/>
+    <mergeCell ref="A26:O26"/>
+    <mergeCell ref="B27:B28"/>
+    <mergeCell ref="D27:F27"/>
+    <mergeCell ref="J27:L27"/>
     <mergeCell ref="A1:O1"/>
     <mergeCell ref="C71:F71"/>
     <mergeCell ref="C14:C15"/>
@@ -2463,45 +2482,30 @@
     <mergeCell ref="M14:O14"/>
     <mergeCell ref="D14:F14"/>
     <mergeCell ref="A13:O13"/>
-    <mergeCell ref="C27:C28"/>
-    <mergeCell ref="J14:L14"/>
-    <mergeCell ref="G27:I27"/>
-    <mergeCell ref="B14:B15"/>
-    <mergeCell ref="A3:O3"/>
-    <mergeCell ref="A27:A28"/>
-    <mergeCell ref="A26:O26"/>
-    <mergeCell ref="B27:B28"/>
-    <mergeCell ref="D27:F27"/>
-    <mergeCell ref="J27:L27"/>
-    <mergeCell ref="A48:O69"/>
-    <mergeCell ref="A45:O46"/>
-    <mergeCell ref="A44:O44"/>
-    <mergeCell ref="A39:O39"/>
-    <mergeCell ref="A40:O42"/>
   </mergeCells>
   <conditionalFormatting sqref="G16:G23">
     <cfRule type="expression" dxfId="5" priority="6" stopIfTrue="1">
       <formula>AND(G16&lt;&gt;"",D16&lt;&gt;"",G16&gt;=1.05*D16)</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="G29:G36">
+    <cfRule type="expression" dxfId="4" priority="3" stopIfTrue="1">
+      <formula>AND(G29&lt;&gt;"",D29&lt;&gt;"",G29&gt;=1.05*D29)</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="J16:J23">
-    <cfRule type="expression" dxfId="4" priority="5" stopIfTrue="1">
+    <cfRule type="expression" dxfId="3" priority="5" stopIfTrue="1">
       <formula>AND(J16&lt;&gt;"",G16&lt;&gt;"",J16&gt;=1.05*G16)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M16:M23">
-    <cfRule type="expression" dxfId="3" priority="4" stopIfTrue="1">
-      <formula>AND(M16&lt;&gt;"",J16&lt;&gt;"",M16&gt;=1.05*J16)</formula>
+  <conditionalFormatting sqref="J29:J36">
+    <cfRule type="expression" dxfId="2" priority="2" stopIfTrue="1">
+      <formula>AND(J29&lt;&gt;"",G29&lt;&gt;"",J29&gt;=1.05*G29)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G29:G36">
-    <cfRule type="expression" dxfId="2" priority="3" stopIfTrue="1">
-      <formula>AND(G29&lt;&gt;"",D29&lt;&gt;"",G29&gt;=1.05*D29)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J29:J36">
-    <cfRule type="expression" dxfId="1" priority="2" stopIfTrue="1">
-      <formula>AND(J29&lt;&gt;"",G29&lt;&gt;"",J29&gt;=1.05*G29)</formula>
+  <conditionalFormatting sqref="M16:M23">
+    <cfRule type="expression" dxfId="1" priority="4" stopIfTrue="1">
+      <formula>AND(M16&lt;&gt;"",J16&lt;&gt;"",M16&gt;=1.05*J16)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M29:M36">

</xml_diff>

<commit_message>
Drie doelregio's per voet; geen maskerexport in de ziekenhuizen
REDCap: e09, e24uc en e24oc met doelregio d1-d3 links en d4-d6 rechts,
zonder zijdeveld; berekende velden en norm_totaal (van zes) mee;
1449 velden, documenten bijgewerkt. eCRF 09 en 24 (alle kopieen): per
voet, met de hielregel. Pressure Monitoring Tool: blok 7 geschrapt,
blokken op Visit en sjabloon "in te vullen door het studieteam", geen
maskerexport meer vermeld; 24b zonder "Multimask". 09b versie 1.4 zonder
blok 7 en zonder de tabel met maskerprogramma's. PARADISE_BRONNEN en
werkpakket1-tijdlijn bijgewerkt.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/(e)CRF/Per nummer/24b_Opvolgtool piekdruk en ontlasting (Novel pedar).xlsx
+++ b/(e)CRF/Per nummer/24b_Opvolgtool piekdruk en ontlasting (Novel pedar).xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://kuleuven-my.sharepoint.com/personal/janou_debuyser_kuleuven_be1/Documents/Documents/PhD Brugge/Site/(e)CRF/Per nummer/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="24" documentId="11_71D650B1929CCFA6FD70D0ED0D1FF050D6CE9E36" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DC9D05F0-9D7A-487C-BCAA-544881AB70D2}"/>
+  <xr:revisionPtr revIDLastSave="26" documentId="11_71D650B1929CCFA6FD70D0ED0D1FF050D6CE9E36" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{554DEA7A-0BC7-4E17-8C96-1B56C3F88DFC}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1560" yWindow="1560" windowWidth="14400" windowHeight="7450" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Opvolgtool" sheetId="1" r:id="rId1"/>
@@ -77,9 +77,6 @@
     <t>V2 / V4 / V6 / V8 (omcirkelen)</t>
   </si>
   <si>
-    <t>Regio (Multimask)</t>
-  </si>
-  <si>
     <t>Doelregio?</t>
   </si>
   <si>
@@ -158,6 +155,9 @@
     <t>Doelregio's per voet: de regio van de vorige voetzweer - altijd, ook onder 200 kPa - plus de twee regio's in voorvoet of middenvoet met de hoogste piekdruk boven 200 kPa zonder zool. De hiel telt alleen mee als daar de vorige voetzweer zat. Beide worden automatisch als DOELREGIO gemarkeerd; de vorige voetzweer kies je bovenaan bij elke voet.
 Norm per doelregio: piekdruk met zool onder 200 kPa, OF minstens 25% lager dan de referentie. De referentie is de meting zonder zool op visite 2 (in-shoe, in hetzelfde schoeisel, zonder de CMFO) en blijft op visite 4, 6 en 8 dezelfde. Noteer op visite 2 de waarde na de laatste aanpassing.
 Is de norm niet gehaald (NEE), of kleurt een piekdruk oranje omdat ze 5% of meer hoger ligt dan de vorige visite, dan wordt de CMFO aangepast volgens eCRF 23 en opnieuw gemeten.</t>
+  </si>
+  <si>
+    <t>Regio</t>
   </si>
 </sst>
 </file>
@@ -472,42 +472,42 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -863,7 +863,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:O71"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
     <col min="2" max="2" width="15" customWidth="1"/>
@@ -878,64 +878,64 @@
     <col min="14" max="15" width="13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="9" t="s">
+    <row r="1" spans="1:15" ht="26.15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="23" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="10"/>
-      <c r="C1" s="10"/>
-      <c r="D1" s="10"/>
-      <c r="E1" s="10"/>
-      <c r="F1" s="10"/>
-      <c r="G1" s="10"/>
-      <c r="H1" s="10"/>
-      <c r="I1" s="10"/>
-      <c r="J1" s="10"/>
-      <c r="K1" s="10"/>
-      <c r="L1" s="10"/>
-      <c r="M1" s="10"/>
-      <c r="N1" s="10"/>
-      <c r="O1" s="10"/>
-    </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A2" s="18" t="s">
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
+      <c r="H1" s="13"/>
+      <c r="I1" s="13"/>
+      <c r="J1" s="13"/>
+      <c r="K1" s="13"/>
+      <c r="L1" s="13"/>
+      <c r="M1" s="13"/>
+      <c r="N1" s="13"/>
+      <c r="O1" s="13"/>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A2" s="30" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="10"/>
-      <c r="C2" s="10"/>
-      <c r="D2" s="10"/>
-      <c r="E2" s="10"/>
-      <c r="F2" s="10"/>
-      <c r="G2" s="10"/>
-      <c r="H2" s="10"/>
-      <c r="I2" s="10"/>
-      <c r="J2" s="10"/>
-      <c r="K2" s="10"/>
-      <c r="L2" s="10"/>
-      <c r="M2" s="10"/>
-      <c r="N2" s="10"/>
-      <c r="O2" s="10"/>
-    </row>
-    <row r="3" spans="1:15" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="20" t="s">
+      <c r="B2" s="13"/>
+      <c r="C2" s="13"/>
+      <c r="D2" s="13"/>
+      <c r="E2" s="13"/>
+      <c r="F2" s="13"/>
+      <c r="G2" s="13"/>
+      <c r="H2" s="13"/>
+      <c r="I2" s="13"/>
+      <c r="J2" s="13"/>
+      <c r="K2" s="13"/>
+      <c r="L2" s="13"/>
+      <c r="M2" s="13"/>
+      <c r="N2" s="13"/>
+      <c r="O2" s="13"/>
+    </row>
+    <row r="3" spans="1:15" ht="28" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="18" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="10"/>
-      <c r="C3" s="10"/>
-      <c r="D3" s="10"/>
-      <c r="E3" s="10"/>
-      <c r="F3" s="10"/>
-      <c r="G3" s="10"/>
-      <c r="H3" s="10"/>
-      <c r="I3" s="10"/>
-      <c r="J3" s="10"/>
-      <c r="K3" s="10"/>
-      <c r="L3" s="10"/>
-      <c r="M3" s="10"/>
-      <c r="N3" s="10"/>
-      <c r="O3" s="10"/>
-    </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="B3" s="13"/>
+      <c r="C3" s="13"/>
+      <c r="D3" s="13"/>
+      <c r="E3" s="13"/>
+      <c r="F3" s="13"/>
+      <c r="G3" s="13"/>
+      <c r="H3" s="13"/>
+      <c r="I3" s="13"/>
+      <c r="J3" s="13"/>
+      <c r="K3" s="13"/>
+      <c r="L3" s="13"/>
+      <c r="M3" s="13"/>
+      <c r="N3" s="13"/>
+      <c r="O3" s="13"/>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
@@ -943,7 +943,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>5</v>
       </c>
@@ -951,7 +951,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>7</v>
       </c>
@@ -961,7 +961,7 @@
       </c>
       <c r="I7" s="2"/>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>9</v>
       </c>
@@ -973,7 +973,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>12</v>
       </c>
@@ -981,119 +981,119 @@
         <v>13</v>
       </c>
     </row>
-    <row r="12" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="15" t="s">
+    <row r="12" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="27" t="s">
+        <v>30</v>
+      </c>
+      <c r="B12" s="27"/>
+      <c r="C12" s="27"/>
+      <c r="D12" s="27"/>
+      <c r="E12" s="28"/>
+      <c r="F12" s="28"/>
+      <c r="G12" s="28"/>
+      <c r="H12" s="29" t="s">
         <v>31</v>
       </c>
-      <c r="B12" s="15"/>
-      <c r="C12" s="15"/>
-      <c r="D12" s="15"/>
-      <c r="E12" s="16"/>
-      <c r="F12" s="16"/>
-      <c r="G12" s="16"/>
-      <c r="H12" s="17" t="s">
+      <c r="I12" s="13"/>
+      <c r="J12" s="13"/>
+      <c r="K12" s="13"/>
+      <c r="L12" s="13"/>
+      <c r="M12" s="13"/>
+      <c r="N12" s="13"/>
+      <c r="O12" s="13"/>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A13" s="22"/>
+      <c r="B13" s="13"/>
+      <c r="C13" s="13"/>
+      <c r="D13" s="13"/>
+      <c r="E13" s="13"/>
+      <c r="F13" s="13"/>
+      <c r="G13" s="13"/>
+      <c r="H13" s="13"/>
+      <c r="I13" s="13"/>
+      <c r="J13" s="13"/>
+      <c r="K13" s="13"/>
+      <c r="L13" s="13"/>
+      <c r="M13" s="13"/>
+      <c r="N13" s="13"/>
+      <c r="O13" s="13"/>
+    </row>
+    <row r="14" spans="1:15" ht="16" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="21" t="s">
+        <v>40</v>
+      </c>
+      <c r="B14" s="21" t="s">
         <v>32</v>
       </c>
-      <c r="I12" s="10"/>
-      <c r="J12" s="10"/>
-      <c r="K12" s="10"/>
-      <c r="L12" s="10"/>
-      <c r="M12" s="10"/>
-      <c r="N12" s="10"/>
-      <c r="O12" s="10"/>
-    </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A13" s="19"/>
-      <c r="B13" s="10"/>
-      <c r="C13" s="10"/>
-      <c r="D13" s="10"/>
-      <c r="E13" s="10"/>
-      <c r="F13" s="10"/>
-      <c r="G13" s="10"/>
-      <c r="H13" s="10"/>
-      <c r="I13" s="10"/>
-      <c r="J13" s="10"/>
-      <c r="K13" s="10"/>
-      <c r="L13" s="10"/>
-      <c r="M13" s="10"/>
-      <c r="N13" s="10"/>
-      <c r="O13" s="10"/>
-    </row>
-    <row r="14" spans="1:15" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="14" t="s">
+      <c r="C14" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="B14" s="14" t="s">
+      <c r="D14" s="21" t="s">
+        <v>15</v>
+      </c>
+      <c r="E14" s="13"/>
+      <c r="F14" s="13"/>
+      <c r="G14" s="21" t="s">
+        <v>16</v>
+      </c>
+      <c r="H14" s="13"/>
+      <c r="I14" s="13"/>
+      <c r="J14" s="21" t="s">
+        <v>17</v>
+      </c>
+      <c r="K14" s="13"/>
+      <c r="L14" s="13"/>
+      <c r="M14" s="21" t="s">
+        <v>18</v>
+      </c>
+      <c r="N14" s="13"/>
+      <c r="O14" s="13"/>
+    </row>
+    <row r="15" spans="1:15" ht="28" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="13"/>
+      <c r="B15" s="13"/>
+      <c r="C15" s="13"/>
+      <c r="D15" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="C14" s="14" t="s">
-        <v>15</v>
-      </c>
-      <c r="D14" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="E14" s="10"/>
-      <c r="F14" s="10"/>
-      <c r="G14" s="14" t="s">
-        <v>17</v>
-      </c>
-      <c r="H14" s="10"/>
-      <c r="I14" s="10"/>
-      <c r="J14" s="14" t="s">
-        <v>18</v>
-      </c>
-      <c r="K14" s="10"/>
-      <c r="L14" s="10"/>
-      <c r="M14" s="14" t="s">
+      <c r="E15" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="F15" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="N14" s="10"/>
-      <c r="O14" s="10"/>
-    </row>
-    <row r="15" spans="1:15" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="10"/>
-      <c r="B15" s="10"/>
-      <c r="C15" s="10"/>
-      <c r="D15" s="3" t="s">
+      <c r="G15" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="H15" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="E15" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="F15" s="3" t="s">
+      <c r="I15" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="J15" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="K15" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="L15" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="M15" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="N15" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="O15" s="3" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A16" s="4" t="s">
         <v>20</v>
-      </c>
-      <c r="G15" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="H15" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="I15" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="J15" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="K15" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="L15" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="M15" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="N15" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="O15" s="3" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A16" s="4" t="s">
-        <v>21</v>
       </c>
       <c r="B16" s="5"/>
       <c r="C16" s="6" t="str">
@@ -1137,13 +1137,13 @@
         <v/>
       </c>
     </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A17" s="4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B17" s="5"/>
       <c r="C17" s="6" t="str">
-        <f>IF($E$12=$A17,"DOELREGIO",IF(B17="","",IF(AND(B17&gt;200,RANK(B17,$B$17:$B$23)&lt;=2),"DOELREGIO","")))</f>
+        <f t="shared" ref="C17:C23" si="8">IF($E$12=$A17,"DOELREGIO",IF(B17="","",IF(AND(B17&gt;200,RANK(B17,$B$17:$B$23)&lt;=2),"DOELREGIO","")))</f>
         <v/>
       </c>
       <c r="D17" s="5"/>
@@ -1183,13 +1183,13 @@
         <v/>
       </c>
     </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A18" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B18" s="5"/>
       <c r="C18" s="6" t="str">
-        <f>IF($E$12=$A18,"DOELREGIO",IF(B18="","",IF(AND(B18&gt;200,RANK(B18,$B$17:$B$23)&lt;=2),"DOELREGIO","")))</f>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="D18" s="5"/>
@@ -1229,13 +1229,13 @@
         <v/>
       </c>
     </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A19" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B19" s="5"/>
       <c r="C19" s="6" t="str">
-        <f>IF($E$12=$A19,"DOELREGIO",IF(B19="","",IF(AND(B19&gt;200,RANK(B19,$B$17:$B$23)&lt;=2),"DOELREGIO","")))</f>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="D19" s="5"/>
@@ -1275,13 +1275,13 @@
         <v/>
       </c>
     </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A20" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B20" s="5"/>
       <c r="C20" s="6" t="str">
-        <f>IF($E$12=$A20,"DOELREGIO",IF(B20="","",IF(AND(B20&gt;200,RANK(B20,$B$17:$B$23)&lt;=2),"DOELREGIO","")))</f>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="D20" s="5"/>
@@ -1321,13 +1321,13 @@
         <v/>
       </c>
     </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A21" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B21" s="5"/>
       <c r="C21" s="6" t="str">
-        <f>IF($E$12=$A21,"DOELREGIO",IF(B21="","",IF(AND(B21&gt;200,RANK(B21,$B$17:$B$23)&lt;=2),"DOELREGIO","")))</f>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="D21" s="5"/>
@@ -1367,13 +1367,13 @@
         <v/>
       </c>
     </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A22" s="4" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B22" s="5"/>
       <c r="C22" s="6" t="str">
-        <f>IF($E$12=$A22,"DOELREGIO",IF(B22="","",IF(AND(B22&gt;200,RANK(B22,$B$17:$B$23)&lt;=2),"DOELREGIO","")))</f>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="D22" s="5"/>
@@ -1413,13 +1413,13 @@
         <v/>
       </c>
     </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A23" s="4" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B23" s="5"/>
       <c r="C23" s="6" t="str">
-        <f>IF($E$12=$A23,"DOELREGIO",IF(B23="","",IF(AND(B23&gt;200,RANK(B23,$B$17:$B$23)&lt;=2),"DOELREGIO","")))</f>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="D23" s="5"/>
@@ -1459,119 +1459,119 @@
         <v/>
       </c>
     </row>
-    <row r="25" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="15" t="s">
-        <v>36</v>
-      </c>
-      <c r="B25" s="15"/>
-      <c r="C25" s="15"/>
-      <c r="D25" s="15"/>
-      <c r="E25" s="16"/>
-      <c r="F25" s="16"/>
-      <c r="G25" s="16"/>
-      <c r="H25" s="17" t="s">
+    <row r="25" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A25" s="27" t="s">
+        <v>35</v>
+      </c>
+      <c r="B25" s="27"/>
+      <c r="C25" s="27"/>
+      <c r="D25" s="27"/>
+      <c r="E25" s="28"/>
+      <c r="F25" s="28"/>
+      <c r="G25" s="28"/>
+      <c r="H25" s="29" t="s">
+        <v>31</v>
+      </c>
+      <c r="I25" s="13"/>
+      <c r="J25" s="13"/>
+      <c r="K25" s="13"/>
+      <c r="L25" s="13"/>
+      <c r="M25" s="13"/>
+      <c r="N25" s="13"/>
+      <c r="O25" s="13"/>
+    </row>
+    <row r="26" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A26" s="22"/>
+      <c r="B26" s="13"/>
+      <c r="C26" s="13"/>
+      <c r="D26" s="13"/>
+      <c r="E26" s="13"/>
+      <c r="F26" s="13"/>
+      <c r="G26" s="13"/>
+      <c r="H26" s="13"/>
+      <c r="I26" s="13"/>
+      <c r="J26" s="13"/>
+      <c r="K26" s="13"/>
+      <c r="L26" s="13"/>
+      <c r="M26" s="13"/>
+      <c r="N26" s="13"/>
+      <c r="O26" s="13"/>
+    </row>
+    <row r="27" spans="1:15" ht="16" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A27" s="21" t="s">
+        <v>40</v>
+      </c>
+      <c r="B27" s="21" t="s">
         <v>32</v>
       </c>
-      <c r="I25" s="10"/>
-      <c r="J25" s="10"/>
-      <c r="K25" s="10"/>
-      <c r="L25" s="10"/>
-      <c r="M25" s="10"/>
-      <c r="N25" s="10"/>
-      <c r="O25" s="10"/>
-    </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A26" s="19"/>
-      <c r="B26" s="10"/>
-      <c r="C26" s="10"/>
-      <c r="D26" s="10"/>
-      <c r="E26" s="10"/>
-      <c r="F26" s="10"/>
-      <c r="G26" s="10"/>
-      <c r="H26" s="10"/>
-      <c r="I26" s="10"/>
-      <c r="J26" s="10"/>
-      <c r="K26" s="10"/>
-      <c r="L26" s="10"/>
-      <c r="M26" s="10"/>
-      <c r="N26" s="10"/>
-      <c r="O26" s="10"/>
-    </row>
-    <row r="27" spans="1:15" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="14" t="s">
+      <c r="C27" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="B27" s="14" t="s">
+      <c r="D27" s="21" t="s">
+        <v>15</v>
+      </c>
+      <c r="E27" s="13"/>
+      <c r="F27" s="13"/>
+      <c r="G27" s="21" t="s">
+        <v>16</v>
+      </c>
+      <c r="H27" s="13"/>
+      <c r="I27" s="13"/>
+      <c r="J27" s="21" t="s">
+        <v>17</v>
+      </c>
+      <c r="K27" s="13"/>
+      <c r="L27" s="13"/>
+      <c r="M27" s="21" t="s">
+        <v>18</v>
+      </c>
+      <c r="N27" s="13"/>
+      <c r="O27" s="13"/>
+    </row>
+    <row r="28" spans="1:15" ht="28" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A28" s="13"/>
+      <c r="B28" s="13"/>
+      <c r="C28" s="13"/>
+      <c r="D28" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="C27" s="14" t="s">
-        <v>15</v>
-      </c>
-      <c r="D27" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="E27" s="10"/>
-      <c r="F27" s="10"/>
-      <c r="G27" s="14" t="s">
-        <v>17</v>
-      </c>
-      <c r="H27" s="10"/>
-      <c r="I27" s="10"/>
-      <c r="J27" s="14" t="s">
-        <v>18</v>
-      </c>
-      <c r="K27" s="10"/>
-      <c r="L27" s="10"/>
-      <c r="M27" s="14" t="s">
+      <c r="E28" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="F28" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="N27" s="10"/>
-      <c r="O27" s="10"/>
-    </row>
-    <row r="28" spans="1:15" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="10"/>
-      <c r="B28" s="10"/>
-      <c r="C28" s="10"/>
-      <c r="D28" s="3" t="s">
+      <c r="G28" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="H28" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="E28" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="F28" s="3" t="s">
+      <c r="I28" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="J28" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="K28" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="L28" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="M28" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="N28" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="O28" s="3" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="29" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A29" s="4" t="s">
         <v>20</v>
-      </c>
-      <c r="G28" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="H28" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="I28" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="J28" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="K28" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="L28" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="M28" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="N28" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="O28" s="3" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="29" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A29" s="4" t="s">
-        <v>21</v>
       </c>
       <c r="B29" s="5"/>
       <c r="C29" s="6" t="str">
@@ -1580,892 +1580,877 @@
       </c>
       <c r="D29" s="5"/>
       <c r="E29" s="6" t="str">
-        <f t="shared" ref="E29:E36" si="8">IF(OR($B29="",D29=""),"",ROUND(($B29-D29)/$B29*100,1))</f>
+        <f t="shared" ref="E29:E36" si="9">IF(OR($B29="",D29=""),"",ROUND(($B29-D29)/$B29*100,1))</f>
         <v/>
       </c>
       <c r="F29" s="7" t="str">
-        <f t="shared" ref="F29:F36" si="9">IF(OR($B29="",D29=""),"",IF(OR(D29&lt;200,($B29-D29)/$B29&gt;=0.25),"JA","NEE"))</f>
+        <f t="shared" ref="F29:F36" si="10">IF(OR($B29="",D29=""),"",IF(OR(D29&lt;200,($B29-D29)/$B29&gt;=0.25),"JA","NEE"))</f>
         <v/>
       </c>
       <c r="G29" s="5"/>
       <c r="H29" s="6" t="str">
-        <f t="shared" ref="H29:H36" si="10">IF(OR($B29="",G29=""),"",ROUND(($B29-G29)/$B29*100,1))</f>
+        <f t="shared" ref="H29:H36" si="11">IF(OR($B29="",G29=""),"",ROUND(($B29-G29)/$B29*100,1))</f>
         <v/>
       </c>
       <c r="I29" s="7" t="str">
-        <f t="shared" ref="I29:I36" si="11">IF(OR($B29="",G29=""),"",IF(OR(G29&lt;200,($B29-G29)/$B29&gt;=0.25),"JA","NEE"))</f>
+        <f t="shared" ref="I29:I36" si="12">IF(OR($B29="",G29=""),"",IF(OR(G29&lt;200,($B29-G29)/$B29&gt;=0.25),"JA","NEE"))</f>
         <v/>
       </c>
       <c r="J29" s="5"/>
       <c r="K29" s="6" t="str">
-        <f t="shared" ref="K29:K36" si="12">IF(OR($B29="",J29=""),"",ROUND(($B29-J29)/$B29*100,1))</f>
+        <f t="shared" ref="K29:K36" si="13">IF(OR($B29="",J29=""),"",ROUND(($B29-J29)/$B29*100,1))</f>
         <v/>
       </c>
       <c r="L29" s="7" t="str">
-        <f t="shared" ref="L29:L36" si="13">IF(OR($B29="",J29=""),"",IF(OR(J29&lt;200,($B29-J29)/$B29&gt;=0.25),"JA","NEE"))</f>
+        <f t="shared" ref="L29:L36" si="14">IF(OR($B29="",J29=""),"",IF(OR(J29&lt;200,($B29-J29)/$B29&gt;=0.25),"JA","NEE"))</f>
         <v/>
       </c>
       <c r="M29" s="5"/>
       <c r="N29" s="6" t="str">
-        <f t="shared" ref="N29:N36" si="14">IF(OR($B29="",M29=""),"",ROUND(($B29-M29)/$B29*100,1))</f>
+        <f t="shared" ref="N29:N36" si="15">IF(OR($B29="",M29=""),"",ROUND(($B29-M29)/$B29*100,1))</f>
         <v/>
       </c>
       <c r="O29" s="7" t="str">
-        <f t="shared" ref="O29:O36" si="15">IF(OR($B29="",M29=""),"",IF(OR(M29&lt;200,($B29-M29)/$B29&gt;=0.25),"JA","NEE"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="30" spans="1:15" x14ac:dyDescent="0.25">
+        <f t="shared" ref="O29:O36" si="16">IF(OR($B29="",M29=""),"",IF(OR(M29&lt;200,($B29-M29)/$B29&gt;=0.25),"JA","NEE"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A30" s="4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B30" s="5"/>
       <c r="C30" s="6" t="str">
-        <f>IF($E$25=$A30,"DOELREGIO",IF(B30="","",IF(AND(B30&gt;200,RANK(B30,$B$30:$B$36)&lt;=2),"DOELREGIO","")))</f>
+        <f t="shared" ref="C30:C36" si="17">IF($E$25=$A30,"DOELREGIO",IF(B30="","",IF(AND(B30&gt;200,RANK(B30,$B$30:$B$36)&lt;=2),"DOELREGIO","")))</f>
         <v/>
       </c>
       <c r="D30" s="5"/>
       <c r="E30" s="6" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="F30" s="7" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="G30" s="5"/>
       <c r="H30" s="6" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="I30" s="7" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J30" s="5"/>
       <c r="K30" s="6" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="L30" s="7" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="M30" s="5"/>
       <c r="N30" s="6" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="O30" s="7" t="str">
-        <f t="shared" si="15"/>
-        <v/>
-      </c>
-    </row>
-    <row r="31" spans="1:15" x14ac:dyDescent="0.25">
+        <f t="shared" si="16"/>
+        <v/>
+      </c>
+    </row>
+    <row r="31" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A31" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B31" s="5"/>
       <c r="C31" s="6" t="str">
-        <f>IF($E$25=$A31,"DOELREGIO",IF(B31="","",IF(AND(B31&gt;200,RANK(B31,$B$30:$B$36)&lt;=2),"DOELREGIO","")))</f>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="D31" s="5"/>
       <c r="E31" s="6" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="F31" s="7" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="G31" s="5"/>
       <c r="H31" s="6" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="I31" s="7" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J31" s="5"/>
       <c r="K31" s="6" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="L31" s="7" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="M31" s="5"/>
       <c r="N31" s="6" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="O31" s="7" t="str">
-        <f t="shared" si="15"/>
-        <v/>
-      </c>
-    </row>
-    <row r="32" spans="1:15" x14ac:dyDescent="0.25">
+        <f t="shared" si="16"/>
+        <v/>
+      </c>
+    </row>
+    <row r="32" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A32" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B32" s="5"/>
       <c r="C32" s="6" t="str">
-        <f>IF($E$25=$A32,"DOELREGIO",IF(B32="","",IF(AND(B32&gt;200,RANK(B32,$B$30:$B$36)&lt;=2),"DOELREGIO","")))</f>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="D32" s="5"/>
       <c r="E32" s="6" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="F32" s="7" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="G32" s="5"/>
       <c r="H32" s="6" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="I32" s="7" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J32" s="5"/>
       <c r="K32" s="6" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="L32" s="7" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="M32" s="5"/>
       <c r="N32" s="6" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="O32" s="7" t="str">
-        <f t="shared" si="15"/>
-        <v/>
-      </c>
-    </row>
-    <row r="33" spans="1:15" x14ac:dyDescent="0.25">
+        <f t="shared" si="16"/>
+        <v/>
+      </c>
+    </row>
+    <row r="33" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A33" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B33" s="5"/>
       <c r="C33" s="6" t="str">
-        <f>IF($E$25=$A33,"DOELREGIO",IF(B33="","",IF(AND(B33&gt;200,RANK(B33,$B$30:$B$36)&lt;=2),"DOELREGIO","")))</f>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="D33" s="5"/>
       <c r="E33" s="6" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="F33" s="7" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="G33" s="5"/>
       <c r="H33" s="6" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="I33" s="7" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J33" s="5"/>
       <c r="K33" s="6" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="L33" s="7" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="M33" s="5"/>
       <c r="N33" s="6" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="O33" s="7" t="str">
-        <f t="shared" si="15"/>
-        <v/>
-      </c>
-    </row>
-    <row r="34" spans="1:15" x14ac:dyDescent="0.25">
+        <f t="shared" si="16"/>
+        <v/>
+      </c>
+    </row>
+    <row r="34" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A34" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B34" s="5"/>
       <c r="C34" s="6" t="str">
-        <f>IF($E$25=$A34,"DOELREGIO",IF(B34="","",IF(AND(B34&gt;200,RANK(B34,$B$30:$B$36)&lt;=2),"DOELREGIO","")))</f>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="D34" s="5"/>
       <c r="E34" s="6" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="F34" s="7" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="G34" s="5"/>
       <c r="H34" s="6" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="I34" s="7" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J34" s="5"/>
       <c r="K34" s="6" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="L34" s="7" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="M34" s="5"/>
       <c r="N34" s="6" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="O34" s="7" t="str">
-        <f t="shared" si="15"/>
-        <v/>
-      </c>
-    </row>
-    <row r="35" spans="1:15" x14ac:dyDescent="0.25">
+        <f t="shared" si="16"/>
+        <v/>
+      </c>
+    </row>
+    <row r="35" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A35" s="4" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B35" s="5"/>
       <c r="C35" s="6" t="str">
-        <f>IF($E$25=$A35,"DOELREGIO",IF(B35="","",IF(AND(B35&gt;200,RANK(B35,$B$30:$B$36)&lt;=2),"DOELREGIO","")))</f>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="D35" s="5"/>
       <c r="E35" s="6" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="F35" s="7" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="G35" s="5"/>
       <c r="H35" s="6" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="I35" s="7" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J35" s="5"/>
       <c r="K35" s="6" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="L35" s="7" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="M35" s="5"/>
       <c r="N35" s="6" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="O35" s="7" t="str">
-        <f t="shared" si="15"/>
-        <v/>
-      </c>
-    </row>
-    <row r="36" spans="1:15" x14ac:dyDescent="0.25">
+        <f t="shared" si="16"/>
+        <v/>
+      </c>
+    </row>
+    <row r="36" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A36" s="4" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B36" s="5"/>
       <c r="C36" s="6" t="str">
-        <f>IF($E$25=$A36,"DOELREGIO",IF(B36="","",IF(AND(B36&gt;200,RANK(B36,$B$30:$B$36)&lt;=2),"DOELREGIO","")))</f>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="D36" s="5"/>
       <c r="E36" s="6" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="F36" s="7" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="G36" s="5"/>
       <c r="H36" s="6" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="I36" s="7" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J36" s="5"/>
       <c r="K36" s="6" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="L36" s="7" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="M36" s="5"/>
       <c r="N36" s="6" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="O36" s="7" t="str">
-        <f t="shared" si="15"/>
-        <v/>
-      </c>
-    </row>
-    <row r="39" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="29" t="s">
+        <f t="shared" si="16"/>
+        <v/>
+      </c>
+    </row>
+    <row r="39" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A39" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="B39" s="13"/>
+      <c r="C39" s="13"/>
+      <c r="D39" s="13"/>
+      <c r="E39" s="13"/>
+      <c r="F39" s="13"/>
+      <c r="G39" s="13"/>
+      <c r="H39" s="13"/>
+      <c r="I39" s="13"/>
+      <c r="J39" s="13"/>
+      <c r="K39" s="13"/>
+      <c r="L39" s="13"/>
+      <c r="M39" s="13"/>
+      <c r="N39" s="13"/>
+      <c r="O39" s="13"/>
+    </row>
+    <row r="40" spans="1:15" ht="90" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A40" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="B40" s="13"/>
+      <c r="C40" s="13"/>
+      <c r="D40" s="13"/>
+      <c r="E40" s="13"/>
+      <c r="F40" s="13"/>
+      <c r="G40" s="13"/>
+      <c r="H40" s="13"/>
+      <c r="I40" s="13"/>
+      <c r="J40" s="13"/>
+      <c r="K40" s="13"/>
+      <c r="L40" s="13"/>
+      <c r="M40" s="13"/>
+      <c r="N40" s="13"/>
+      <c r="O40" s="13"/>
+    </row>
+    <row r="41" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A41" s="13"/>
+      <c r="B41" s="13"/>
+      <c r="C41" s="13"/>
+      <c r="D41" s="13"/>
+      <c r="E41" s="13"/>
+      <c r="F41" s="13"/>
+      <c r="G41" s="13"/>
+      <c r="H41" s="13"/>
+      <c r="I41" s="13"/>
+      <c r="J41" s="13"/>
+      <c r="K41" s="13"/>
+      <c r="L41" s="13"/>
+      <c r="M41" s="13"/>
+      <c r="N41" s="13"/>
+      <c r="O41" s="13"/>
+    </row>
+    <row r="42" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A42" s="13"/>
+      <c r="B42" s="13"/>
+      <c r="C42" s="13"/>
+      <c r="D42" s="13"/>
+      <c r="E42" s="13"/>
+      <c r="F42" s="13"/>
+      <c r="G42" s="13"/>
+      <c r="H42" s="13"/>
+      <c r="I42" s="13"/>
+      <c r="J42" s="13"/>
+      <c r="K42" s="13"/>
+      <c r="L42" s="13"/>
+      <c r="M42" s="13"/>
+      <c r="N42" s="13"/>
+      <c r="O42" s="13"/>
+    </row>
+    <row r="44" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A44" s="19" t="s">
+        <v>36</v>
+      </c>
+      <c r="B44" s="13"/>
+      <c r="C44" s="13"/>
+      <c r="D44" s="13"/>
+      <c r="E44" s="13"/>
+      <c r="F44" s="13"/>
+      <c r="G44" s="13"/>
+      <c r="H44" s="13"/>
+      <c r="I44" s="13"/>
+      <c r="J44" s="13"/>
+      <c r="K44" s="13"/>
+      <c r="L44" s="13"/>
+      <c r="M44" s="13"/>
+      <c r="N44" s="13"/>
+      <c r="O44" s="13"/>
+    </row>
+    <row r="45" spans="1:15" ht="16" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A45" s="18" t="s">
+        <v>37</v>
+      </c>
+      <c r="B45" s="13"/>
+      <c r="C45" s="13"/>
+      <c r="D45" s="13"/>
+      <c r="E45" s="13"/>
+      <c r="F45" s="13"/>
+      <c r="G45" s="13"/>
+      <c r="H45" s="13"/>
+      <c r="I45" s="13"/>
+      <c r="J45" s="13"/>
+      <c r="K45" s="13"/>
+      <c r="L45" s="13"/>
+      <c r="M45" s="13"/>
+      <c r="N45" s="13"/>
+      <c r="O45" s="13"/>
+    </row>
+    <row r="46" spans="1:15" ht="16" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A46" s="13"/>
+      <c r="B46" s="13"/>
+      <c r="C46" s="13"/>
+      <c r="D46" s="13"/>
+      <c r="E46" s="13"/>
+      <c r="F46" s="13"/>
+      <c r="G46" s="13"/>
+      <c r="H46" s="13"/>
+      <c r="I46" s="13"/>
+      <c r="J46" s="13"/>
+      <c r="K46" s="13"/>
+      <c r="L46" s="13"/>
+      <c r="M46" s="13"/>
+      <c r="N46" s="13"/>
+      <c r="O46" s="13"/>
+    </row>
+    <row r="48" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A48" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="B48" s="10"/>
+      <c r="C48" s="10"/>
+      <c r="D48" s="10"/>
+      <c r="E48" s="10"/>
+      <c r="F48" s="10"/>
+      <c r="G48" s="10"/>
+      <c r="H48" s="10"/>
+      <c r="I48" s="10"/>
+      <c r="J48" s="10"/>
+      <c r="K48" s="10"/>
+      <c r="L48" s="10"/>
+      <c r="M48" s="10"/>
+      <c r="N48" s="10"/>
+      <c r="O48" s="11"/>
+    </row>
+    <row r="49" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A49" s="12"/>
+      <c r="B49" s="13"/>
+      <c r="C49" s="13"/>
+      <c r="D49" s="13"/>
+      <c r="E49" s="13"/>
+      <c r="F49" s="13"/>
+      <c r="G49" s="13"/>
+      <c r="H49" s="13"/>
+      <c r="I49" s="13"/>
+      <c r="J49" s="13"/>
+      <c r="K49" s="13"/>
+      <c r="L49" s="13"/>
+      <c r="M49" s="13"/>
+      <c r="N49" s="13"/>
+      <c r="O49" s="14"/>
+    </row>
+    <row r="50" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A50" s="12"/>
+      <c r="B50" s="13"/>
+      <c r="C50" s="13"/>
+      <c r="D50" s="13"/>
+      <c r="E50" s="13"/>
+      <c r="F50" s="13"/>
+      <c r="G50" s="13"/>
+      <c r="H50" s="13"/>
+      <c r="I50" s="13"/>
+      <c r="J50" s="13"/>
+      <c r="K50" s="13"/>
+      <c r="L50" s="13"/>
+      <c r="M50" s="13"/>
+      <c r="N50" s="13"/>
+      <c r="O50" s="14"/>
+    </row>
+    <row r="51" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A51" s="12"/>
+      <c r="B51" s="13"/>
+      <c r="C51" s="13"/>
+      <c r="D51" s="13"/>
+      <c r="E51" s="13"/>
+      <c r="F51" s="13"/>
+      <c r="G51" s="13"/>
+      <c r="H51" s="13"/>
+      <c r="I51" s="13"/>
+      <c r="J51" s="13"/>
+      <c r="K51" s="13"/>
+      <c r="L51" s="13"/>
+      <c r="M51" s="13"/>
+      <c r="N51" s="13"/>
+      <c r="O51" s="14"/>
+    </row>
+    <row r="52" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A52" s="12"/>
+      <c r="B52" s="13"/>
+      <c r="C52" s="13"/>
+      <c r="D52" s="13"/>
+      <c r="E52" s="13"/>
+      <c r="F52" s="13"/>
+      <c r="G52" s="13"/>
+      <c r="H52" s="13"/>
+      <c r="I52" s="13"/>
+      <c r="J52" s="13"/>
+      <c r="K52" s="13"/>
+      <c r="L52" s="13"/>
+      <c r="M52" s="13"/>
+      <c r="N52" s="13"/>
+      <c r="O52" s="14"/>
+    </row>
+    <row r="53" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A53" s="12"/>
+      <c r="B53" s="13"/>
+      <c r="C53" s="13"/>
+      <c r="D53" s="13"/>
+      <c r="E53" s="13"/>
+      <c r="F53" s="13"/>
+      <c r="G53" s="13"/>
+      <c r="H53" s="13"/>
+      <c r="I53" s="13"/>
+      <c r="J53" s="13"/>
+      <c r="K53" s="13"/>
+      <c r="L53" s="13"/>
+      <c r="M53" s="13"/>
+      <c r="N53" s="13"/>
+      <c r="O53" s="14"/>
+    </row>
+    <row r="54" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A54" s="12"/>
+      <c r="B54" s="13"/>
+      <c r="C54" s="13"/>
+      <c r="D54" s="13"/>
+      <c r="E54" s="13"/>
+      <c r="F54" s="13"/>
+      <c r="G54" s="13"/>
+      <c r="H54" s="13"/>
+      <c r="I54" s="13"/>
+      <c r="J54" s="13"/>
+      <c r="K54" s="13"/>
+      <c r="L54" s="13"/>
+      <c r="M54" s="13"/>
+      <c r="N54" s="13"/>
+      <c r="O54" s="14"/>
+    </row>
+    <row r="55" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A55" s="12"/>
+      <c r="B55" s="13"/>
+      <c r="C55" s="13"/>
+      <c r="D55" s="13"/>
+      <c r="E55" s="13"/>
+      <c r="F55" s="13"/>
+      <c r="G55" s="13"/>
+      <c r="H55" s="13"/>
+      <c r="I55" s="13"/>
+      <c r="J55" s="13"/>
+      <c r="K55" s="13"/>
+      <c r="L55" s="13"/>
+      <c r="M55" s="13"/>
+      <c r="N55" s="13"/>
+      <c r="O55" s="14"/>
+    </row>
+    <row r="56" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A56" s="12"/>
+      <c r="B56" s="13"/>
+      <c r="C56" s="13"/>
+      <c r="D56" s="13"/>
+      <c r="E56" s="13"/>
+      <c r="F56" s="13"/>
+      <c r="G56" s="13"/>
+      <c r="H56" s="13"/>
+      <c r="I56" s="13"/>
+      <c r="J56" s="13"/>
+      <c r="K56" s="13"/>
+      <c r="L56" s="13"/>
+      <c r="M56" s="13"/>
+      <c r="N56" s="13"/>
+      <c r="O56" s="14"/>
+    </row>
+    <row r="57" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A57" s="12"/>
+      <c r="B57" s="13"/>
+      <c r="C57" s="13"/>
+      <c r="D57" s="13"/>
+      <c r="E57" s="13"/>
+      <c r="F57" s="13"/>
+      <c r="G57" s="13"/>
+      <c r="H57" s="13"/>
+      <c r="I57" s="13"/>
+      <c r="J57" s="13"/>
+      <c r="K57" s="13"/>
+      <c r="L57" s="13"/>
+      <c r="M57" s="13"/>
+      <c r="N57" s="13"/>
+      <c r="O57" s="14"/>
+    </row>
+    <row r="58" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A58" s="12"/>
+      <c r="B58" s="13"/>
+      <c r="C58" s="13"/>
+      <c r="D58" s="13"/>
+      <c r="E58" s="13"/>
+      <c r="F58" s="13"/>
+      <c r="G58" s="13"/>
+      <c r="H58" s="13"/>
+      <c r="I58" s="13"/>
+      <c r="J58" s="13"/>
+      <c r="K58" s="13"/>
+      <c r="L58" s="13"/>
+      <c r="M58" s="13"/>
+      <c r="N58" s="13"/>
+      <c r="O58" s="14"/>
+    </row>
+    <row r="59" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A59" s="12"/>
+      <c r="B59" s="13"/>
+      <c r="C59" s="13"/>
+      <c r="D59" s="13"/>
+      <c r="E59" s="13"/>
+      <c r="F59" s="13"/>
+      <c r="G59" s="13"/>
+      <c r="H59" s="13"/>
+      <c r="I59" s="13"/>
+      <c r="J59" s="13"/>
+      <c r="K59" s="13"/>
+      <c r="L59" s="13"/>
+      <c r="M59" s="13"/>
+      <c r="N59" s="13"/>
+      <c r="O59" s="14"/>
+    </row>
+    <row r="60" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A60" s="12"/>
+      <c r="B60" s="13"/>
+      <c r="C60" s="13"/>
+      <c r="D60" s="13"/>
+      <c r="E60" s="13"/>
+      <c r="F60" s="13"/>
+      <c r="G60" s="13"/>
+      <c r="H60" s="13"/>
+      <c r="I60" s="13"/>
+      <c r="J60" s="13"/>
+      <c r="K60" s="13"/>
+      <c r="L60" s="13"/>
+      <c r="M60" s="13"/>
+      <c r="N60" s="13"/>
+      <c r="O60" s="14"/>
+    </row>
+    <row r="61" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A61" s="12"/>
+      <c r="B61" s="13"/>
+      <c r="C61" s="13"/>
+      <c r="D61" s="13"/>
+      <c r="E61" s="13"/>
+      <c r="F61" s="13"/>
+      <c r="G61" s="13"/>
+      <c r="H61" s="13"/>
+      <c r="I61" s="13"/>
+      <c r="J61" s="13"/>
+      <c r="K61" s="13"/>
+      <c r="L61" s="13"/>
+      <c r="M61" s="13"/>
+      <c r="N61" s="13"/>
+      <c r="O61" s="14"/>
+    </row>
+    <row r="62" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A62" s="12"/>
+      <c r="B62" s="13"/>
+      <c r="C62" s="13"/>
+      <c r="D62" s="13"/>
+      <c r="E62" s="13"/>
+      <c r="F62" s="13"/>
+      <c r="G62" s="13"/>
+      <c r="H62" s="13"/>
+      <c r="I62" s="13"/>
+      <c r="J62" s="13"/>
+      <c r="K62" s="13"/>
+      <c r="L62" s="13"/>
+      <c r="M62" s="13"/>
+      <c r="N62" s="13"/>
+      <c r="O62" s="14"/>
+    </row>
+    <row r="63" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A63" s="12"/>
+      <c r="B63" s="13"/>
+      <c r="C63" s="13"/>
+      <c r="D63" s="13"/>
+      <c r="E63" s="13"/>
+      <c r="F63" s="13"/>
+      <c r="G63" s="13"/>
+      <c r="H63" s="13"/>
+      <c r="I63" s="13"/>
+      <c r="J63" s="13"/>
+      <c r="K63" s="13"/>
+      <c r="L63" s="13"/>
+      <c r="M63" s="13"/>
+      <c r="N63" s="13"/>
+      <c r="O63" s="14"/>
+    </row>
+    <row r="64" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A64" s="12"/>
+      <c r="B64" s="13"/>
+      <c r="C64" s="13"/>
+      <c r="D64" s="13"/>
+      <c r="E64" s="13"/>
+      <c r="F64" s="13"/>
+      <c r="G64" s="13"/>
+      <c r="H64" s="13"/>
+      <c r="I64" s="13"/>
+      <c r="J64" s="13"/>
+      <c r="K64" s="13"/>
+      <c r="L64" s="13"/>
+      <c r="M64" s="13"/>
+      <c r="N64" s="13"/>
+      <c r="O64" s="14"/>
+    </row>
+    <row r="65" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A65" s="12"/>
+      <c r="B65" s="13"/>
+      <c r="C65" s="13"/>
+      <c r="D65" s="13"/>
+      <c r="E65" s="13"/>
+      <c r="F65" s="13"/>
+      <c r="G65" s="13"/>
+      <c r="H65" s="13"/>
+      <c r="I65" s="13"/>
+      <c r="J65" s="13"/>
+      <c r="K65" s="13"/>
+      <c r="L65" s="13"/>
+      <c r="M65" s="13"/>
+      <c r="N65" s="13"/>
+      <c r="O65" s="14"/>
+    </row>
+    <row r="66" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A66" s="12"/>
+      <c r="B66" s="13"/>
+      <c r="C66" s="13"/>
+      <c r="D66" s="13"/>
+      <c r="E66" s="13"/>
+      <c r="F66" s="13"/>
+      <c r="G66" s="13"/>
+      <c r="H66" s="13"/>
+      <c r="I66" s="13"/>
+      <c r="J66" s="13"/>
+      <c r="K66" s="13"/>
+      <c r="L66" s="13"/>
+      <c r="M66" s="13"/>
+      <c r="N66" s="13"/>
+      <c r="O66" s="14"/>
+    </row>
+    <row r="67" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A67" s="12"/>
+      <c r="B67" s="13"/>
+      <c r="C67" s="13"/>
+      <c r="D67" s="13"/>
+      <c r="E67" s="13"/>
+      <c r="F67" s="13"/>
+      <c r="G67" s="13"/>
+      <c r="H67" s="13"/>
+      <c r="I67" s="13"/>
+      <c r="J67" s="13"/>
+      <c r="K67" s="13"/>
+      <c r="L67" s="13"/>
+      <c r="M67" s="13"/>
+      <c r="N67" s="13"/>
+      <c r="O67" s="14"/>
+    </row>
+    <row r="68" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A68" s="12"/>
+      <c r="B68" s="13"/>
+      <c r="C68" s="13"/>
+      <c r="D68" s="13"/>
+      <c r="E68" s="13"/>
+      <c r="F68" s="13"/>
+      <c r="G68" s="13"/>
+      <c r="H68" s="13"/>
+      <c r="I68" s="13"/>
+      <c r="J68" s="13"/>
+      <c r="K68" s="13"/>
+      <c r="L68" s="13"/>
+      <c r="M68" s="13"/>
+      <c r="N68" s="13"/>
+      <c r="O68" s="14"/>
+    </row>
+    <row r="69" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A69" s="15"/>
+      <c r="B69" s="16"/>
+      <c r="C69" s="16"/>
+      <c r="D69" s="16"/>
+      <c r="E69" s="16"/>
+      <c r="F69" s="16"/>
+      <c r="G69" s="16"/>
+      <c r="H69" s="16"/>
+      <c r="I69" s="16"/>
+      <c r="J69" s="16"/>
+      <c r="K69" s="16"/>
+      <c r="L69" s="16"/>
+      <c r="M69" s="16"/>
+      <c r="N69" s="16"/>
+      <c r="O69" s="17"/>
+    </row>
+    <row r="71" spans="1:15" ht="16" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A71" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="B39" s="10"/>
-      <c r="C39" s="10"/>
-      <c r="D39" s="10"/>
-      <c r="E39" s="10"/>
-      <c r="F39" s="10"/>
-      <c r="G39" s="10"/>
-      <c r="H39" s="10"/>
-      <c r="I39" s="10"/>
-      <c r="J39" s="10"/>
-      <c r="K39" s="10"/>
-      <c r="L39" s="10"/>
-      <c r="M39" s="10"/>
-      <c r="N39" s="10"/>
-      <c r="O39" s="10"/>
-    </row>
-    <row r="40" spans="1:15" ht="90" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="30" t="s">
-        <v>40</v>
-      </c>
-      <c r="B40" s="10"/>
-      <c r="C40" s="10"/>
-      <c r="D40" s="10"/>
-      <c r="E40" s="10"/>
-      <c r="F40" s="10"/>
-      <c r="G40" s="10"/>
-      <c r="H40" s="10"/>
-      <c r="I40" s="10"/>
-      <c r="J40" s="10"/>
-      <c r="K40" s="10"/>
-      <c r="L40" s="10"/>
-      <c r="M40" s="10"/>
-      <c r="N40" s="10"/>
-      <c r="O40" s="10"/>
-    </row>
-    <row r="41" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A41" s="10"/>
-      <c r="B41" s="10"/>
-      <c r="C41" s="10"/>
-      <c r="D41" s="10"/>
-      <c r="E41" s="10"/>
-      <c r="F41" s="10"/>
-      <c r="G41" s="10"/>
-      <c r="H41" s="10"/>
-      <c r="I41" s="10"/>
-      <c r="J41" s="10"/>
-      <c r="K41" s="10"/>
-      <c r="L41" s="10"/>
-      <c r="M41" s="10"/>
-      <c r="N41" s="10"/>
-      <c r="O41" s="10"/>
-    </row>
-    <row r="42" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A42" s="10"/>
-      <c r="B42" s="10"/>
-      <c r="C42" s="10"/>
-      <c r="D42" s="10"/>
-      <c r="E42" s="10"/>
-      <c r="F42" s="10"/>
-      <c r="G42" s="10"/>
-      <c r="H42" s="10"/>
-      <c r="I42" s="10"/>
-      <c r="J42" s="10"/>
-      <c r="K42" s="10"/>
-      <c r="L42" s="10"/>
-      <c r="M42" s="10"/>
-      <c r="N42" s="10"/>
-      <c r="O42" s="10"/>
-    </row>
-    <row r="44" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="29" t="s">
-        <v>37</v>
-      </c>
-      <c r="B44" s="10"/>
-      <c r="C44" s="10"/>
-      <c r="D44" s="10"/>
-      <c r="E44" s="10"/>
-      <c r="F44" s="10"/>
-      <c r="G44" s="10"/>
-      <c r="H44" s="10"/>
-      <c r="I44" s="10"/>
-      <c r="J44" s="10"/>
-      <c r="K44" s="10"/>
-      <c r="L44" s="10"/>
-      <c r="M44" s="10"/>
-      <c r="N44" s="10"/>
-      <c r="O44" s="10"/>
-    </row>
-    <row r="45" spans="1:15" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="20" t="s">
-        <v>38</v>
-      </c>
-      <c r="B45" s="10"/>
-      <c r="C45" s="10"/>
-      <c r="D45" s="10"/>
-      <c r="E45" s="10"/>
-      <c r="F45" s="10"/>
-      <c r="G45" s="10"/>
-      <c r="H45" s="10"/>
-      <c r="I45" s="10"/>
-      <c r="J45" s="10"/>
-      <c r="K45" s="10"/>
-      <c r="L45" s="10"/>
-      <c r="M45" s="10"/>
-      <c r="N45" s="10"/>
-      <c r="O45" s="10"/>
-    </row>
-    <row r="46" spans="1:15" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="10"/>
-      <c r="B46" s="10"/>
-      <c r="C46" s="10"/>
-      <c r="D46" s="10"/>
-      <c r="E46" s="10"/>
-      <c r="F46" s="10"/>
-      <c r="G46" s="10"/>
-      <c r="H46" s="10"/>
-      <c r="I46" s="10"/>
-      <c r="J46" s="10"/>
-      <c r="K46" s="10"/>
-      <c r="L46" s="10"/>
-      <c r="M46" s="10"/>
-      <c r="N46" s="10"/>
-      <c r="O46" s="10"/>
-    </row>
-    <row r="48" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A48" s="21" t="s">
-        <v>39</v>
-      </c>
-      <c r="B48" s="22"/>
-      <c r="C48" s="22"/>
-      <c r="D48" s="22"/>
-      <c r="E48" s="22"/>
-      <c r="F48" s="22"/>
-      <c r="G48" s="22"/>
-      <c r="H48" s="22"/>
-      <c r="I48" s="22"/>
-      <c r="J48" s="22"/>
-      <c r="K48" s="22"/>
-      <c r="L48" s="22"/>
-      <c r="M48" s="22"/>
-      <c r="N48" s="22"/>
-      <c r="O48" s="23"/>
-    </row>
-    <row r="49" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A49" s="24"/>
-      <c r="B49" s="10"/>
-      <c r="C49" s="10"/>
-      <c r="D49" s="10"/>
-      <c r="E49" s="10"/>
-      <c r="F49" s="10"/>
-      <c r="G49" s="10"/>
-      <c r="H49" s="10"/>
-      <c r="I49" s="10"/>
-      <c r="J49" s="10"/>
-      <c r="K49" s="10"/>
-      <c r="L49" s="10"/>
-      <c r="M49" s="10"/>
-      <c r="N49" s="10"/>
-      <c r="O49" s="25"/>
-    </row>
-    <row r="50" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A50" s="24"/>
-      <c r="B50" s="10"/>
-      <c r="C50" s="10"/>
-      <c r="D50" s="10"/>
-      <c r="E50" s="10"/>
-      <c r="F50" s="10"/>
-      <c r="G50" s="10"/>
-      <c r="H50" s="10"/>
-      <c r="I50" s="10"/>
-      <c r="J50" s="10"/>
-      <c r="K50" s="10"/>
-      <c r="L50" s="10"/>
-      <c r="M50" s="10"/>
-      <c r="N50" s="10"/>
-      <c r="O50" s="25"/>
-    </row>
-    <row r="51" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A51" s="24"/>
-      <c r="B51" s="10"/>
-      <c r="C51" s="10"/>
-      <c r="D51" s="10"/>
-      <c r="E51" s="10"/>
-      <c r="F51" s="10"/>
-      <c r="G51" s="10"/>
-      <c r="H51" s="10"/>
-      <c r="I51" s="10"/>
-      <c r="J51" s="10"/>
-      <c r="K51" s="10"/>
-      <c r="L51" s="10"/>
-      <c r="M51" s="10"/>
-      <c r="N51" s="10"/>
-      <c r="O51" s="25"/>
-    </row>
-    <row r="52" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A52" s="24"/>
-      <c r="B52" s="10"/>
-      <c r="C52" s="10"/>
-      <c r="D52" s="10"/>
-      <c r="E52" s="10"/>
-      <c r="F52" s="10"/>
-      <c r="G52" s="10"/>
-      <c r="H52" s="10"/>
-      <c r="I52" s="10"/>
-      <c r="J52" s="10"/>
-      <c r="K52" s="10"/>
-      <c r="L52" s="10"/>
-      <c r="M52" s="10"/>
-      <c r="N52" s="10"/>
-      <c r="O52" s="25"/>
-    </row>
-    <row r="53" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A53" s="24"/>
-      <c r="B53" s="10"/>
-      <c r="C53" s="10"/>
-      <c r="D53" s="10"/>
-      <c r="E53" s="10"/>
-      <c r="F53" s="10"/>
-      <c r="G53" s="10"/>
-      <c r="H53" s="10"/>
-      <c r="I53" s="10"/>
-      <c r="J53" s="10"/>
-      <c r="K53" s="10"/>
-      <c r="L53" s="10"/>
-      <c r="M53" s="10"/>
-      <c r="N53" s="10"/>
-      <c r="O53" s="25"/>
-    </row>
-    <row r="54" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A54" s="24"/>
-      <c r="B54" s="10"/>
-      <c r="C54" s="10"/>
-      <c r="D54" s="10"/>
-      <c r="E54" s="10"/>
-      <c r="F54" s="10"/>
-      <c r="G54" s="10"/>
-      <c r="H54" s="10"/>
-      <c r="I54" s="10"/>
-      <c r="J54" s="10"/>
-      <c r="K54" s="10"/>
-      <c r="L54" s="10"/>
-      <c r="M54" s="10"/>
-      <c r="N54" s="10"/>
-      <c r="O54" s="25"/>
-    </row>
-    <row r="55" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A55" s="24"/>
-      <c r="B55" s="10"/>
-      <c r="C55" s="10"/>
-      <c r="D55" s="10"/>
-      <c r="E55" s="10"/>
-      <c r="F55" s="10"/>
-      <c r="G55" s="10"/>
-      <c r="H55" s="10"/>
-      <c r="I55" s="10"/>
-      <c r="J55" s="10"/>
-      <c r="K55" s="10"/>
-      <c r="L55" s="10"/>
-      <c r="M55" s="10"/>
-      <c r="N55" s="10"/>
-      <c r="O55" s="25"/>
-    </row>
-    <row r="56" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A56" s="24"/>
-      <c r="B56" s="10"/>
-      <c r="C56" s="10"/>
-      <c r="D56" s="10"/>
-      <c r="E56" s="10"/>
-      <c r="F56" s="10"/>
-      <c r="G56" s="10"/>
-      <c r="H56" s="10"/>
-      <c r="I56" s="10"/>
-      <c r="J56" s="10"/>
-      <c r="K56" s="10"/>
-      <c r="L56" s="10"/>
-      <c r="M56" s="10"/>
-      <c r="N56" s="10"/>
-      <c r="O56" s="25"/>
-    </row>
-    <row r="57" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A57" s="24"/>
-      <c r="B57" s="10"/>
-      <c r="C57" s="10"/>
-      <c r="D57" s="10"/>
-      <c r="E57" s="10"/>
-      <c r="F57" s="10"/>
-      <c r="G57" s="10"/>
-      <c r="H57" s="10"/>
-      <c r="I57" s="10"/>
-      <c r="J57" s="10"/>
-      <c r="K57" s="10"/>
-      <c r="L57" s="10"/>
-      <c r="M57" s="10"/>
-      <c r="N57" s="10"/>
-      <c r="O57" s="25"/>
-    </row>
-    <row r="58" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A58" s="24"/>
-      <c r="B58" s="10"/>
-      <c r="C58" s="10"/>
-      <c r="D58" s="10"/>
-      <c r="E58" s="10"/>
-      <c r="F58" s="10"/>
-      <c r="G58" s="10"/>
-      <c r="H58" s="10"/>
-      <c r="I58" s="10"/>
-      <c r="J58" s="10"/>
-      <c r="K58" s="10"/>
-      <c r="L58" s="10"/>
-      <c r="M58" s="10"/>
-      <c r="N58" s="10"/>
-      <c r="O58" s="25"/>
-    </row>
-    <row r="59" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A59" s="24"/>
-      <c r="B59" s="10"/>
-      <c r="C59" s="10"/>
-      <c r="D59" s="10"/>
-      <c r="E59" s="10"/>
-      <c r="F59" s="10"/>
-      <c r="G59" s="10"/>
-      <c r="H59" s="10"/>
-      <c r="I59" s="10"/>
-      <c r="J59" s="10"/>
-      <c r="K59" s="10"/>
-      <c r="L59" s="10"/>
-      <c r="M59" s="10"/>
-      <c r="N59" s="10"/>
-      <c r="O59" s="25"/>
-    </row>
-    <row r="60" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A60" s="24"/>
-      <c r="B60" s="10"/>
-      <c r="C60" s="10"/>
-      <c r="D60" s="10"/>
-      <c r="E60" s="10"/>
-      <c r="F60" s="10"/>
-      <c r="G60" s="10"/>
-      <c r="H60" s="10"/>
-      <c r="I60" s="10"/>
-      <c r="J60" s="10"/>
-      <c r="K60" s="10"/>
-      <c r="L60" s="10"/>
-      <c r="M60" s="10"/>
-      <c r="N60" s="10"/>
-      <c r="O60" s="25"/>
-    </row>
-    <row r="61" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A61" s="24"/>
-      <c r="B61" s="10"/>
-      <c r="C61" s="10"/>
-      <c r="D61" s="10"/>
-      <c r="E61" s="10"/>
-      <c r="F61" s="10"/>
-      <c r="G61" s="10"/>
-      <c r="H61" s="10"/>
-      <c r="I61" s="10"/>
-      <c r="J61" s="10"/>
-      <c r="K61" s="10"/>
-      <c r="L61" s="10"/>
-      <c r="M61" s="10"/>
-      <c r="N61" s="10"/>
-      <c r="O61" s="25"/>
-    </row>
-    <row r="62" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A62" s="24"/>
-      <c r="B62" s="10"/>
-      <c r="C62" s="10"/>
-      <c r="D62" s="10"/>
-      <c r="E62" s="10"/>
-      <c r="F62" s="10"/>
-      <c r="G62" s="10"/>
-      <c r="H62" s="10"/>
-      <c r="I62" s="10"/>
-      <c r="J62" s="10"/>
-      <c r="K62" s="10"/>
-      <c r="L62" s="10"/>
-      <c r="M62" s="10"/>
-      <c r="N62" s="10"/>
-      <c r="O62" s="25"/>
-    </row>
-    <row r="63" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A63" s="24"/>
-      <c r="B63" s="10"/>
-      <c r="C63" s="10"/>
-      <c r="D63" s="10"/>
-      <c r="E63" s="10"/>
-      <c r="F63" s="10"/>
-      <c r="G63" s="10"/>
-      <c r="H63" s="10"/>
-      <c r="I63" s="10"/>
-      <c r="J63" s="10"/>
-      <c r="K63" s="10"/>
-      <c r="L63" s="10"/>
-      <c r="M63" s="10"/>
-      <c r="N63" s="10"/>
-      <c r="O63" s="25"/>
-    </row>
-    <row r="64" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A64" s="24"/>
-      <c r="B64" s="10"/>
-      <c r="C64" s="10"/>
-      <c r="D64" s="10"/>
-      <c r="E64" s="10"/>
-      <c r="F64" s="10"/>
-      <c r="G64" s="10"/>
-      <c r="H64" s="10"/>
-      <c r="I64" s="10"/>
-      <c r="J64" s="10"/>
-      <c r="K64" s="10"/>
-      <c r="L64" s="10"/>
-      <c r="M64" s="10"/>
-      <c r="N64" s="10"/>
-      <c r="O64" s="25"/>
-    </row>
-    <row r="65" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A65" s="24"/>
-      <c r="B65" s="10"/>
-      <c r="C65" s="10"/>
-      <c r="D65" s="10"/>
-      <c r="E65" s="10"/>
-      <c r="F65" s="10"/>
-      <c r="G65" s="10"/>
-      <c r="H65" s="10"/>
-      <c r="I65" s="10"/>
-      <c r="J65" s="10"/>
-      <c r="K65" s="10"/>
-      <c r="L65" s="10"/>
-      <c r="M65" s="10"/>
-      <c r="N65" s="10"/>
-      <c r="O65" s="25"/>
-    </row>
-    <row r="66" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A66" s="24"/>
-      <c r="B66" s="10"/>
-      <c r="C66" s="10"/>
-      <c r="D66" s="10"/>
-      <c r="E66" s="10"/>
-      <c r="F66" s="10"/>
-      <c r="G66" s="10"/>
-      <c r="H66" s="10"/>
-      <c r="I66" s="10"/>
-      <c r="J66" s="10"/>
-      <c r="K66" s="10"/>
-      <c r="L66" s="10"/>
-      <c r="M66" s="10"/>
-      <c r="N66" s="10"/>
-      <c r="O66" s="25"/>
-    </row>
-    <row r="67" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A67" s="24"/>
-      <c r="B67" s="10"/>
-      <c r="C67" s="10"/>
-      <c r="D67" s="10"/>
-      <c r="E67" s="10"/>
-      <c r="F67" s="10"/>
-      <c r="G67" s="10"/>
-      <c r="H67" s="10"/>
-      <c r="I67" s="10"/>
-      <c r="J67" s="10"/>
-      <c r="K67" s="10"/>
-      <c r="L67" s="10"/>
-      <c r="M67" s="10"/>
-      <c r="N67" s="10"/>
-      <c r="O67" s="25"/>
-    </row>
-    <row r="68" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A68" s="24"/>
-      <c r="B68" s="10"/>
-      <c r="C68" s="10"/>
-      <c r="D68" s="10"/>
-      <c r="E68" s="10"/>
-      <c r="F68" s="10"/>
-      <c r="G68" s="10"/>
-      <c r="H68" s="10"/>
-      <c r="I68" s="10"/>
-      <c r="J68" s="10"/>
-      <c r="K68" s="10"/>
-      <c r="L68" s="10"/>
-      <c r="M68" s="10"/>
-      <c r="N68" s="10"/>
-      <c r="O68" s="25"/>
-    </row>
-    <row r="69" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A69" s="26"/>
-      <c r="B69" s="27"/>
-      <c r="C69" s="27"/>
-      <c r="D69" s="27"/>
-      <c r="E69" s="27"/>
-      <c r="F69" s="27"/>
-      <c r="G69" s="27"/>
-      <c r="H69" s="27"/>
-      <c r="I69" s="27"/>
-      <c r="J69" s="27"/>
-      <c r="K69" s="27"/>
-      <c r="L69" s="27"/>
-      <c r="M69" s="27"/>
-      <c r="N69" s="27"/>
-      <c r="O69" s="28"/>
-    </row>
-    <row r="71" spans="1:15" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A71" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="C71" s="11"/>
-      <c r="D71" s="12"/>
-      <c r="E71" s="12"/>
-      <c r="F71" s="13"/>
+      <c r="C71" s="24"/>
+      <c r="D71" s="25"/>
+      <c r="E71" s="25"/>
+      <c r="F71" s="26"/>
     </row>
   </sheetData>
   <mergeCells count="31">
-    <mergeCell ref="A48:O69"/>
-    <mergeCell ref="A45:O46"/>
-    <mergeCell ref="A44:O44"/>
-    <mergeCell ref="A39:O39"/>
-    <mergeCell ref="A40:O42"/>
-    <mergeCell ref="C27:C28"/>
-    <mergeCell ref="J14:L14"/>
-    <mergeCell ref="G27:I27"/>
-    <mergeCell ref="B14:B15"/>
-    <mergeCell ref="A3:O3"/>
-    <mergeCell ref="A27:A28"/>
-    <mergeCell ref="A26:O26"/>
-    <mergeCell ref="B27:B28"/>
-    <mergeCell ref="D27:F27"/>
-    <mergeCell ref="J27:L27"/>
     <mergeCell ref="A1:O1"/>
     <mergeCell ref="C71:F71"/>
     <mergeCell ref="C14:C15"/>
@@ -2482,6 +2467,21 @@
     <mergeCell ref="M14:O14"/>
     <mergeCell ref="D14:F14"/>
     <mergeCell ref="A13:O13"/>
+    <mergeCell ref="C27:C28"/>
+    <mergeCell ref="J14:L14"/>
+    <mergeCell ref="G27:I27"/>
+    <mergeCell ref="B14:B15"/>
+    <mergeCell ref="A3:O3"/>
+    <mergeCell ref="A27:A28"/>
+    <mergeCell ref="A26:O26"/>
+    <mergeCell ref="B27:B28"/>
+    <mergeCell ref="D27:F27"/>
+    <mergeCell ref="J27:L27"/>
+    <mergeCell ref="A48:O69"/>
+    <mergeCell ref="A45:O46"/>
+    <mergeCell ref="A44:O44"/>
+    <mergeCell ref="A39:O39"/>
+    <mergeCell ref="A40:O42"/>
   </mergeCells>
   <conditionalFormatting sqref="G16:G23">
     <cfRule type="expression" dxfId="5" priority="6" stopIfTrue="1">

</xml_diff>